<commit_message>
Corrige estrutura dos arquivos por Seção/Divisão/Grupo pra bater com a referência
Validei cabeçalho a cabeçalho contra os arquivos de Imperatriz em
prjeto_vetor_municipal/planilhas/. Achei e corrigi duas divergências:

- Faltava uma linha em branco entre a nota e o cabeçalho (header estava
  na linha 3, deveria estar na linha 4) nos arquivos Empregos_por_X,
  Empresas_por_X e Renda_por_X.
- A nota de rodapé não mencionava o nível do QL ("QL calculado no nível
  de Seção/Divisão/Grupo") nos arquivos Empregos_por_X e Empresas_por_X.
- A aba "QL Geral" do QL_Grupo_Empresas_por_Porte também estava sem a
  linha em branco antes do cabeçalho.

Ajustei data_loader.py (offset de leitura) de acordo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Empregos_por_Secao_CNAE_RAIS_Ananindeua.xlsx
+++ b/Empregos_por_Secao_CNAE_RAIS_Ananindeua.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF24"/>
+  <dimension ref="A1:AF25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -469,793 +469,689 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Vínculos empregatícios ativos em 31/12. Fonte: RAIS/MTE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Seção</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Nome Seção</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2001</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2003</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2005</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2007</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2009</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2011</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2013</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2015</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2017</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2019</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2021</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2023</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>Emp. 2025</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2001</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2003</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2005</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2007</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2009</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2011</t>
-        </is>
-      </c>
-      <c r="V3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2013</t>
-        </is>
-      </c>
-      <c r="W3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2015</t>
-        </is>
-      </c>
-      <c r="X3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2017</t>
-        </is>
-      </c>
-      <c r="Y3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2019</t>
-        </is>
-      </c>
-      <c r="Z3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2021</t>
-        </is>
-      </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2023</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr">
-        <is>
-          <t>QL 2025</t>
-        </is>
-      </c>
-      <c r="AC3" s="2" t="inlineStr">
-        <is>
-          <t>QL Médio</t>
-        </is>
-      </c>
-      <c r="AD3" s="2" t="inlineStr">
-        <is>
-          <t>Representat. (%)</t>
-        </is>
-      </c>
-      <c r="AE3" s="2" t="inlineStr">
-        <is>
-          <t>Cresc. 5 anos (%)</t>
-        </is>
-      </c>
-      <c r="AF3" s="2" t="inlineStr">
-        <is>
-          <t>Consistência (0-12)</t>
+          <t>Vínculos empregatícios ativos em 31/12. QL calculado no nível de Seção. Fonte: RAIS/MTE.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>AGRICULTURA, PECUÁRIA, PRODUÇÃO FLORESTAL, PESCA E AQÜICULTURA</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>200</v>
-      </c>
-      <c r="D4" t="n">
-        <v>136</v>
-      </c>
-      <c r="E4" t="n">
-        <v>102</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1876</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1506</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1522</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1334</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1715</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1990</v>
-      </c>
-      <c r="L4" t="n">
-        <v>2144</v>
-      </c>
-      <c r="M4" t="n">
-        <v>2286</v>
-      </c>
-      <c r="N4" t="n">
-        <v>181</v>
-      </c>
-      <c r="O4" t="n">
-        <v>190</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.219934</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.087952</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.047489</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0.702551</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0.630103</v>
-      </c>
-      <c r="U4" t="n">
-        <v>0.521001</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.445373</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.541066</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0.6203650000000001</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0.889655</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0.864854</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>0.058522</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>0.065429</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>0.438023</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0.209887</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>-91.13806</v>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>7/12</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Seção</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Nome Seção</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2001</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2003</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2005</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2007</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2009</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2011</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2013</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2015</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2017</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2019</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2021</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2023</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Emp. 2025</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2001</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2003</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2005</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2007</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2009</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2011</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2013</t>
+        </is>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2015</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2017</t>
+        </is>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2019</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2021</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2023</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>QL 2025</t>
+        </is>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>QL Médio</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>Representat. (%)</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>Cresc. 5 anos (%)</t>
+        </is>
+      </c>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>Consistência (0-12)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>INDÚSTRIAS EXTRATIVAS</t>
+          <t>AGRICULTURA, PECUÁRIA, PRODUÇÃO FLORESTAL, PESCA E AQÜICULTURA</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>96</v>
+        <v>200</v>
       </c>
       <c r="D5" t="n">
-        <v>85</v>
+        <v>136</v>
       </c>
       <c r="E5" t="n">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="F5" t="n">
-        <v>160</v>
+        <v>1876</v>
       </c>
       <c r="G5" t="n">
-        <v>120</v>
+        <v>1506</v>
       </c>
       <c r="H5" t="n">
-        <v>99</v>
+        <v>1522</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1334</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1715</v>
       </c>
       <c r="K5" t="n">
-        <v>4</v>
+        <v>1990</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>2144</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>2286</v>
       </c>
       <c r="N5" t="n">
-        <v>2</v>
+        <v>181</v>
       </c>
       <c r="O5" t="n">
-        <v>37</v>
+        <v>190</v>
       </c>
       <c r="P5" t="n">
-        <v>0.569169</v>
+        <v>0.219934</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.323031</v>
+        <v>0.087952</v>
       </c>
       <c r="R5" t="n">
-        <v>0.157789</v>
+        <v>0.047489</v>
       </c>
       <c r="S5" t="n">
-        <v>0.262257</v>
+        <v>0.702551</v>
       </c>
       <c r="T5" t="n">
-        <v>0.180862</v>
+        <v>0.630103</v>
       </c>
       <c r="U5" t="n">
-        <v>0.108343</v>
+        <v>0.521001</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>0.445373</v>
       </c>
       <c r="W5" t="n">
-        <v>0</v>
+        <v>0.541066</v>
       </c>
       <c r="X5" t="n">
-        <v>0.003342</v>
+        <v>0.6203650000000001</v>
       </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>0.889655</v>
       </c>
       <c r="Z5" t="n">
-        <v>0</v>
+        <v>0.864854</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.002574</v>
+        <v>0.058522</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.045367</v>
+        <v>0.065429</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.127133</v>
+        <v>0.438023</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.040873</v>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.209887</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>-91.13806</v>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>4/12</t>
+          <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>INDÚSTRIAS DE TRANSFORMAÇÃO</t>
+          <t>INDÚSTRIAS EXTRATIVAS</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6174</v>
+        <v>96</v>
       </c>
       <c r="D6" t="n">
-        <v>7517</v>
+        <v>85</v>
       </c>
       <c r="E6" t="n">
-        <v>8592</v>
+        <v>59</v>
       </c>
       <c r="F6" t="n">
-        <v>5535</v>
+        <v>160</v>
       </c>
       <c r="G6" t="n">
-        <v>4902</v>
+        <v>120</v>
       </c>
       <c r="H6" t="n">
-        <v>5454</v>
+        <v>99</v>
       </c>
       <c r="I6" t="n">
-        <v>5291</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>5383</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>5330</v>
+        <v>4</v>
       </c>
       <c r="L6" t="n">
-        <v>5946</v>
+        <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>6521</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>8729</v>
+        <v>2</v>
       </c>
       <c r="O6" t="n">
-        <v>9889</v>
+        <v>37</v>
       </c>
       <c r="P6" t="n">
-        <v>1.87852</v>
+        <v>0.569169</v>
       </c>
       <c r="Q6" t="n">
-        <v>1.665559</v>
+        <v>0.323031</v>
       </c>
       <c r="R6" t="n">
-        <v>1.470426</v>
+        <v>0.157789</v>
       </c>
       <c r="S6" t="n">
-        <v>1.329939</v>
+        <v>0.262257</v>
       </c>
       <c r="T6" t="n">
-        <v>1.298055</v>
+        <v>0.180862</v>
       </c>
       <c r="U6" t="n">
-        <v>1.366357</v>
+        <v>0.108343</v>
       </c>
       <c r="V6" t="n">
-        <v>1.347573</v>
+        <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>1.269484</v>
+        <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>1.272711</v>
+        <v>0.003342</v>
       </c>
       <c r="Y6" t="n">
-        <v>1.043302</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>1.013227</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.238425</v>
+        <v>0.002574</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.298093</v>
+        <v>0.045367</v>
       </c>
       <c r="AC6" t="n">
-        <v>1.345513</v>
+        <v>0.127133</v>
       </c>
       <c r="AD6" t="n">
-        <v>10.924054</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>66.31348800000001</v>
+        <v>0.040873</v>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>8/12</t>
+          <t>4/12</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ELETRICIDADE E GÁS</t>
+          <t>INDÚSTRIAS DE TRANSFORMAÇÃO</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>6174</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>7517</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>8592</v>
       </c>
       <c r="F7" t="n">
-        <v>142</v>
+        <v>5535</v>
       </c>
       <c r="G7" t="n">
-        <v>152</v>
+        <v>4902</v>
       </c>
       <c r="H7" t="n">
-        <v>23</v>
+        <v>5454</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>5291</v>
       </c>
       <c r="J7" t="n">
-        <v>14</v>
+        <v>5383</v>
       </c>
       <c r="K7" t="n">
-        <v>14</v>
+        <v>5330</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>5946</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>6521</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>8729</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>9889</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1.87852</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.042232</v>
+        <v>1.665559</v>
       </c>
       <c r="R7" t="n">
-        <v>0.028148</v>
+        <v>1.470426</v>
       </c>
       <c r="S7" t="n">
-        <v>0.836732</v>
+        <v>1.329939</v>
       </c>
       <c r="T7" t="n">
-        <v>1.140237</v>
+        <v>1.298055</v>
       </c>
       <c r="U7" t="n">
-        <v>0.145961</v>
+        <v>1.366357</v>
       </c>
       <c r="V7" t="n">
-        <v>0.006051</v>
+        <v>1.347573</v>
       </c>
       <c r="W7" t="n">
-        <v>0.076768</v>
+        <v>1.269484</v>
       </c>
       <c r="X7" t="n">
-        <v>0.087432</v>
+        <v>1.272711</v>
       </c>
       <c r="Y7" t="n">
-        <v>0</v>
+        <v>1.043302</v>
       </c>
       <c r="Z7" t="n">
-        <v>0</v>
+        <v>1.013227</v>
       </c>
       <c r="AA7" t="n">
-        <v>0</v>
+        <v>1.238425</v>
       </c>
       <c r="AB7" t="n">
-        <v>0</v>
+        <v>1.298093</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.181812</v>
+        <v>1.345513</v>
       </c>
       <c r="AD7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>10.924054</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>66.31348800000001</v>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>4/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ÁGUA, ESGOTO, ATIVIDADES DE GESTÃO DE RESÍDUOS E DESCONTAMINAÇÃO</t>
+          <t>ELETRICIDADE E GÁS</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="E8" t="n">
-        <v>202</v>
+        <v>6</v>
       </c>
       <c r="F8" t="n">
-        <v>124</v>
+        <v>142</v>
       </c>
       <c r="G8" t="n">
-        <v>249</v>
+        <v>152</v>
       </c>
       <c r="H8" t="n">
-        <v>126</v>
+        <v>23</v>
       </c>
       <c r="I8" t="n">
-        <v>325</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>300</v>
+        <v>14</v>
       </c>
       <c r="K8" t="n">
-        <v>446</v>
+        <v>14</v>
       </c>
       <c r="L8" t="n">
-        <v>563</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>583</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>1555</v>
+        <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>1460</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>0.238892</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.649322</v>
+        <v>0.042232</v>
       </c>
       <c r="R8" t="n">
-        <v>1.418067</v>
+        <v>0.028148</v>
       </c>
       <c r="S8" t="n">
-        <v>0.472557</v>
+        <v>0.836732</v>
       </c>
       <c r="T8" t="n">
-        <v>0.708214</v>
+        <v>1.140237</v>
       </c>
       <c r="U8" t="n">
-        <v>0.476449</v>
+        <v>0.145961</v>
       </c>
       <c r="V8" t="n">
-        <v>1.082969</v>
+        <v>0.006051</v>
       </c>
       <c r="W8" t="n">
-        <v>0.917736</v>
+        <v>0.076768</v>
       </c>
       <c r="X8" t="n">
-        <v>1.328189</v>
+        <v>0.087432</v>
       </c>
       <c r="Y8" t="n">
-        <v>1.463911</v>
+        <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>1.311045</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>3.101239</v>
+        <v>0</v>
       </c>
       <c r="AB8" t="n">
-        <v>2.635</v>
+        <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.215661</v>
+        <v>0.181812</v>
       </c>
       <c r="AD8" t="n">
-        <v>1.612814</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>159.325044</v>
+        <v>0</v>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>8/12</t>
+          <t>4/12</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CONSTRUÇÃO</t>
+          <t>ÁGUA, ESGOTO, ATIVIDADES DE GESTÃO DE RESÍDUOS E DESCONTAMINAÇÃO</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2056</v>
+        <v>37</v>
       </c>
       <c r="D9" t="n">
-        <v>2163</v>
+        <v>128</v>
       </c>
       <c r="E9" t="n">
-        <v>2795</v>
+        <v>202</v>
       </c>
       <c r="F9" t="n">
-        <v>4621</v>
+        <v>124</v>
       </c>
       <c r="G9" t="n">
-        <v>5775</v>
+        <v>249</v>
       </c>
       <c r="H9" t="n">
-        <v>7692</v>
+        <v>126</v>
       </c>
       <c r="I9" t="n">
-        <v>6616</v>
+        <v>325</v>
       </c>
       <c r="J9" t="n">
-        <v>7046</v>
+        <v>300</v>
       </c>
       <c r="K9" t="n">
-        <v>7388</v>
+        <v>446</v>
       </c>
       <c r="L9" t="n">
-        <v>5530</v>
+        <v>563</v>
       </c>
       <c r="M9" t="n">
-        <v>4956</v>
+        <v>583</v>
       </c>
       <c r="N9" t="n">
-        <v>6845</v>
+        <v>1555</v>
       </c>
       <c r="O9" t="n">
-        <v>5365</v>
+        <v>1460</v>
       </c>
       <c r="P9" t="n">
-        <v>1.274695</v>
+        <v>0.238892</v>
       </c>
       <c r="Q9" t="n">
-        <v>1.529866</v>
+        <v>0.649322</v>
       </c>
       <c r="R9" t="n">
-        <v>1.335262</v>
+        <v>1.418067</v>
       </c>
       <c r="S9" t="n">
-        <v>1.520138</v>
+        <v>0.472557</v>
       </c>
       <c r="T9" t="n">
-        <v>1.81171</v>
+        <v>0.708214</v>
       </c>
       <c r="U9" t="n">
-        <v>1.630957</v>
+        <v>0.476449</v>
       </c>
       <c r="V9" t="n">
-        <v>1.083491</v>
+        <v>1.082969</v>
       </c>
       <c r="W9" t="n">
-        <v>1.286973</v>
+        <v>0.917736</v>
       </c>
       <c r="X9" t="n">
-        <v>2.037857</v>
+        <v>1.328189</v>
       </c>
       <c r="Y9" t="n">
-        <v>2.010576</v>
+        <v>1.463911</v>
       </c>
       <c r="Z9" t="n">
-        <v>1.472667</v>
+        <v>1.311045</v>
       </c>
       <c r="AA9" t="n">
-        <v>1.664924</v>
+        <v>3.101239</v>
       </c>
       <c r="AB9" t="n">
-        <v>1.311461</v>
+        <v>2.635</v>
       </c>
       <c r="AC9" t="n">
-        <v>1.536198</v>
+        <v>1.215661</v>
       </c>
       <c r="AD9" t="n">
-        <v>5.92654</v>
+        <v>1.612814</v>
       </c>
       <c r="AE9" t="n">
-        <v>-2.983725</v>
+        <v>159.325044</v>
       </c>
       <c r="AF9" t="inlineStr">
         <is>
@@ -1266,724 +1162,724 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>COMÉRCIO; REPARAÇÃO DE VEÍCULOS AUTOMOTORES E MOTOCICLETAS</t>
+          <t>CONSTRUÇÃO</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7415</v>
+        <v>2056</v>
       </c>
       <c r="D10" t="n">
-        <v>10376</v>
+        <v>2163</v>
       </c>
       <c r="E10" t="n">
-        <v>13460</v>
+        <v>2795</v>
       </c>
       <c r="F10" t="n">
-        <v>14277</v>
+        <v>4621</v>
       </c>
       <c r="G10" t="n">
-        <v>14786</v>
+        <v>5775</v>
       </c>
       <c r="H10" t="n">
-        <v>17373</v>
+        <v>7692</v>
       </c>
       <c r="I10" t="n">
-        <v>18382</v>
+        <v>6616</v>
       </c>
       <c r="J10" t="n">
-        <v>18780</v>
+        <v>7046</v>
       </c>
       <c r="K10" t="n">
-        <v>18207</v>
+        <v>7388</v>
       </c>
       <c r="L10" t="n">
-        <v>17599</v>
+        <v>5530</v>
       </c>
       <c r="M10" t="n">
-        <v>20723</v>
+        <v>4956</v>
       </c>
       <c r="N10" t="n">
-        <v>22298</v>
+        <v>6845</v>
       </c>
       <c r="O10" t="n">
-        <v>23853</v>
+        <v>5365</v>
       </c>
       <c r="P10" t="n">
-        <v>1.691867</v>
+        <v>1.274695</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.736383</v>
+        <v>1.529866</v>
       </c>
       <c r="R10" t="n">
-        <v>1.664573</v>
+        <v>1.335262</v>
       </c>
       <c r="S10" t="n">
-        <v>1.602888</v>
+        <v>1.520138</v>
       </c>
       <c r="T10" t="n">
-        <v>1.632403</v>
+        <v>1.81171</v>
       </c>
       <c r="U10" t="n">
-        <v>1.610082</v>
+        <v>1.630957</v>
       </c>
       <c r="V10" t="n">
-        <v>1.583657</v>
+        <v>1.083491</v>
       </c>
       <c r="W10" t="n">
-        <v>1.485592</v>
+        <v>1.286973</v>
       </c>
       <c r="X10" t="n">
-        <v>1.509385</v>
+        <v>2.037857</v>
       </c>
       <c r="Y10" t="n">
-        <v>1.407752</v>
+        <v>2.010576</v>
       </c>
       <c r="Z10" t="n">
-        <v>1.511553</v>
+        <v>1.472667</v>
       </c>
       <c r="AA10" t="n">
-        <v>1.51523</v>
+        <v>1.664924</v>
       </c>
       <c r="AB10" t="n">
-        <v>1.558071</v>
+        <v>1.311461</v>
       </c>
       <c r="AC10" t="n">
-        <v>1.577649</v>
+        <v>1.536198</v>
       </c>
       <c r="AD10" t="n">
-        <v>26.349627</v>
+        <v>5.92654</v>
       </c>
       <c r="AE10" t="n">
-        <v>35.53611</v>
+        <v>-2.983725</v>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TRANSPORTE, ARMAZENAGEM E CORREIO</t>
+          <t>COMÉRCIO; REPARAÇÃO DE VEÍCULOS AUTOMOTORES E MOTOCICLETAS</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4418</v>
+        <v>7415</v>
       </c>
       <c r="D11" t="n">
-        <v>4814</v>
+        <v>10376</v>
       </c>
       <c r="E11" t="n">
-        <v>5331</v>
+        <v>13460</v>
       </c>
       <c r="F11" t="n">
-        <v>5231</v>
+        <v>14277</v>
       </c>
       <c r="G11" t="n">
-        <v>5270</v>
+        <v>14786</v>
       </c>
       <c r="H11" t="n">
-        <v>6493</v>
+        <v>17373</v>
       </c>
       <c r="I11" t="n">
-        <v>6571</v>
+        <v>18382</v>
       </c>
       <c r="J11" t="n">
-        <v>7691</v>
+        <v>18780</v>
       </c>
       <c r="K11" t="n">
-        <v>6630</v>
+        <v>18207</v>
       </c>
       <c r="L11" t="n">
-        <v>6074</v>
+        <v>17599</v>
       </c>
       <c r="M11" t="n">
-        <v>5855</v>
+        <v>20723</v>
       </c>
       <c r="N11" t="n">
-        <v>6645</v>
+        <v>22298</v>
       </c>
       <c r="O11" t="n">
-        <v>6576</v>
+        <v>23853</v>
       </c>
       <c r="P11" t="n">
-        <v>3.555985</v>
+        <v>1.691867</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.432463</v>
+        <v>1.736383</v>
       </c>
       <c r="R11" t="n">
-        <v>3.071248</v>
+        <v>1.664573</v>
       </c>
       <c r="S11" t="n">
-        <v>2.716455</v>
+        <v>1.602888</v>
       </c>
       <c r="T11" t="n">
-        <v>2.744492</v>
+        <v>1.632403</v>
       </c>
       <c r="U11" t="n">
-        <v>2.803307</v>
+        <v>1.610082</v>
       </c>
       <c r="V11" t="n">
-        <v>2.836888</v>
+        <v>1.583657</v>
       </c>
       <c r="W11" t="n">
-        <v>2.898363</v>
+        <v>1.485592</v>
       </c>
       <c r="X11" t="n">
-        <v>2.597792</v>
+        <v>1.509385</v>
       </c>
       <c r="Y11" t="n">
-        <v>2.332161</v>
+        <v>1.407752</v>
       </c>
       <c r="Z11" t="n">
-        <v>2.103383</v>
+        <v>1.511553</v>
       </c>
       <c r="AA11" t="n">
-        <v>2.147584</v>
+        <v>1.51523</v>
       </c>
       <c r="AB11" t="n">
-        <v>2.010303</v>
+        <v>1.558071</v>
       </c>
       <c r="AC11" t="n">
-        <v>2.711571</v>
+        <v>1.577649</v>
       </c>
       <c r="AD11" t="n">
-        <v>7.264292</v>
+        <v>26.349627</v>
       </c>
       <c r="AE11" t="n">
-        <v>8.264735</v>
+        <v>35.53611</v>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>7/12</t>
+          <t>10/12</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ALOJAMENTO E ALIMENTAÇÃO</t>
+          <t>TRANSPORTE, ARMAZENAGEM E CORREIO</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>401</v>
+        <v>4418</v>
       </c>
       <c r="D12" t="n">
-        <v>936</v>
+        <v>4814</v>
       </c>
       <c r="E12" t="n">
-        <v>1093</v>
+        <v>5331</v>
       </c>
       <c r="F12" t="n">
-        <v>1516</v>
+        <v>5231</v>
       </c>
       <c r="G12" t="n">
-        <v>1511</v>
+        <v>5270</v>
       </c>
       <c r="H12" t="n">
-        <v>1961</v>
+        <v>6493</v>
       </c>
       <c r="I12" t="n">
-        <v>1322</v>
+        <v>6571</v>
       </c>
       <c r="J12" t="n">
-        <v>1338</v>
+        <v>7691</v>
       </c>
       <c r="K12" t="n">
-        <v>1577</v>
+        <v>6630</v>
       </c>
       <c r="L12" t="n">
-        <v>1620</v>
+        <v>6074</v>
       </c>
       <c r="M12" t="n">
-        <v>1900</v>
+        <v>5855</v>
       </c>
       <c r="N12" t="n">
-        <v>2563</v>
+        <v>6645</v>
       </c>
       <c r="O12" t="n">
-        <v>2767</v>
+        <v>6576</v>
       </c>
       <c r="P12" t="n">
-        <v>1.049922</v>
+        <v>3.555985</v>
       </c>
       <c r="Q12" t="n">
-        <v>1.331174</v>
+        <v>3.432463</v>
       </c>
       <c r="R12" t="n">
-        <v>1.253481</v>
+        <v>3.071248</v>
       </c>
       <c r="S12" t="n">
-        <v>1.420617</v>
+        <v>2.716455</v>
       </c>
       <c r="T12" t="n">
-        <v>1.30352</v>
+        <v>2.744492</v>
       </c>
       <c r="U12" t="n">
-        <v>1.400883</v>
+        <v>2.803307</v>
       </c>
       <c r="V12" t="n">
-        <v>0.856169</v>
+        <v>2.836888</v>
       </c>
       <c r="W12" t="n">
-        <v>0.793826</v>
+        <v>2.898363</v>
       </c>
       <c r="X12" t="n">
-        <v>1.06089</v>
+        <v>2.597792</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.948354</v>
+        <v>2.332161</v>
       </c>
       <c r="Z12" t="n">
-        <v>1.12726</v>
+        <v>2.103383</v>
       </c>
       <c r="AA12" t="n">
-        <v>1.182529</v>
+        <v>2.147584</v>
       </c>
       <c r="AB12" t="n">
-        <v>1.13324</v>
+        <v>2.010303</v>
       </c>
       <c r="AC12" t="n">
-        <v>1.14322</v>
+        <v>2.711571</v>
       </c>
       <c r="AD12" t="n">
-        <v>3.056614</v>
+        <v>7.264292</v>
       </c>
       <c r="AE12" t="n">
-        <v>70.802469</v>
+        <v>8.264735</v>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>I</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INFORMAÇÃO E COMUNICAÇÃO</t>
+          <t>ALOJAMENTO E ALIMENTAÇÃO</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14</v>
+        <v>401</v>
       </c>
       <c r="D13" t="n">
-        <v>14</v>
+        <v>936</v>
       </c>
       <c r="E13" t="n">
-        <v>47</v>
+        <v>1093</v>
       </c>
       <c r="F13" t="n">
-        <v>43</v>
+        <v>1516</v>
       </c>
       <c r="G13" t="n">
-        <v>35</v>
+        <v>1511</v>
       </c>
       <c r="H13" t="n">
-        <v>33</v>
+        <v>1961</v>
       </c>
       <c r="I13" t="n">
-        <v>73</v>
+        <v>1322</v>
       </c>
       <c r="J13" t="n">
-        <v>125</v>
+        <v>1338</v>
       </c>
       <c r="K13" t="n">
-        <v>223</v>
+        <v>1577</v>
       </c>
       <c r="L13" t="n">
-        <v>259</v>
+        <v>1620</v>
       </c>
       <c r="M13" t="n">
-        <v>240</v>
+        <v>1900</v>
       </c>
       <c r="N13" t="n">
-        <v>536</v>
+        <v>2563</v>
       </c>
       <c r="O13" t="n">
-        <v>568</v>
+        <v>2767</v>
       </c>
       <c r="P13" t="n">
-        <v>0.046888</v>
+        <v>1.049922</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.043606</v>
+        <v>1.331174</v>
       </c>
       <c r="R13" t="n">
-        <v>0.116161</v>
+        <v>1.253481</v>
       </c>
       <c r="S13" t="n">
-        <v>0.118684</v>
+        <v>1.420617</v>
       </c>
       <c r="T13" t="n">
-        <v>0.116535</v>
+        <v>1.30352</v>
       </c>
       <c r="U13" t="n">
-        <v>0.08903800000000001</v>
+        <v>1.400883</v>
       </c>
       <c r="V13" t="n">
-        <v>0.182388</v>
+        <v>0.856169</v>
       </c>
       <c r="W13" t="n">
-        <v>0.244342</v>
+        <v>0.793826</v>
       </c>
       <c r="X13" t="n">
-        <v>0.365163</v>
+        <v>1.06089</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.396953</v>
+        <v>0.948354</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.325877</v>
+        <v>1.12726</v>
       </c>
       <c r="AA13" t="n">
-        <v>0.611114</v>
+        <v>1.182529</v>
       </c>
       <c r="AB13" t="n">
-        <v>0.594433</v>
+        <v>1.13324</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.250091</v>
+        <v>1.14322</v>
       </c>
       <c r="AD13" t="n">
-        <v>0.627451</v>
+        <v>3.056614</v>
       </c>
       <c r="AE13" t="n">
-        <v>119.305019</v>
+        <v>70.802469</v>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>7/12</t>
+          <t>10/12</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>J</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ATIVIDADES FINANCEIRAS, DE SEGUROS E SERVIÇOS RELACIONADOS</t>
+          <t>INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>180</v>
+        <v>14</v>
       </c>
       <c r="D14" t="n">
-        <v>271</v>
+        <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>247</v>
+        <v>47</v>
       </c>
       <c r="F14" t="n">
-        <v>344</v>
+        <v>43</v>
       </c>
       <c r="G14" t="n">
-        <v>351</v>
+        <v>35</v>
       </c>
       <c r="H14" t="n">
-        <v>393</v>
+        <v>33</v>
       </c>
       <c r="I14" t="n">
-        <v>300</v>
+        <v>73</v>
       </c>
       <c r="J14" t="n">
-        <v>376</v>
+        <v>125</v>
       </c>
       <c r="K14" t="n">
-        <v>394</v>
+        <v>223</v>
       </c>
       <c r="L14" t="n">
-        <v>1079</v>
+        <v>259</v>
       </c>
       <c r="M14" t="n">
-        <v>1026</v>
+        <v>240</v>
       </c>
       <c r="N14" t="n">
-        <v>1352</v>
+        <v>536</v>
       </c>
       <c r="O14" t="n">
-        <v>1329</v>
+        <v>568</v>
       </c>
       <c r="P14" t="n">
-        <v>0.43906</v>
+        <v>0.046888</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.561616</v>
+        <v>0.043606</v>
       </c>
       <c r="R14" t="n">
-        <v>0.420777</v>
+        <v>0.116161</v>
       </c>
       <c r="S14" t="n">
-        <v>0.604287</v>
+        <v>0.118684</v>
       </c>
       <c r="T14" t="n">
-        <v>0.5342519999999999</v>
+        <v>0.116535</v>
       </c>
       <c r="U14" t="n">
-        <v>0.576542</v>
+        <v>0.08903800000000001</v>
       </c>
       <c r="V14" t="n">
-        <v>0.429629</v>
+        <v>0.182388</v>
       </c>
       <c r="W14" t="n">
-        <v>0.476789</v>
+        <v>0.244342</v>
       </c>
       <c r="X14" t="n">
-        <v>0.489959</v>
+        <v>0.365163</v>
       </c>
       <c r="Y14" t="n">
-        <v>1.421805</v>
+        <v>0.396953</v>
       </c>
       <c r="Z14" t="n">
-        <v>1.176143</v>
+        <v>0.325877</v>
       </c>
       <c r="AA14" t="n">
-        <v>1.448214</v>
+        <v>0.611114</v>
       </c>
       <c r="AB14" t="n">
-        <v>1.496248</v>
+        <v>0.594433</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.775025</v>
+        <v>0.250091</v>
       </c>
       <c r="AD14" t="n">
-        <v>1.468103</v>
+        <v>0.627451</v>
       </c>
       <c r="AE14" t="n">
-        <v>23.169601</v>
+        <v>119.305019</v>
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>8/12</t>
+          <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>K</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ATIVIDADES IMOBILIÁRIAS</t>
+          <t>ATIVIDADES FINANCEIRAS, DE SEGUROS E SERVIÇOS RELACIONADOS</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>271</v>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>247</v>
       </c>
       <c r="F15" t="n">
-        <v>31</v>
+        <v>344</v>
       </c>
       <c r="G15" t="n">
-        <v>17</v>
+        <v>351</v>
       </c>
       <c r="H15" t="n">
-        <v>76</v>
+        <v>393</v>
       </c>
       <c r="I15" t="n">
-        <v>25</v>
+        <v>300</v>
       </c>
       <c r="J15" t="n">
-        <v>40</v>
+        <v>376</v>
       </c>
       <c r="K15" t="n">
-        <v>180</v>
+        <v>394</v>
       </c>
       <c r="L15" t="n">
-        <v>251</v>
+        <v>1079</v>
       </c>
       <c r="M15" t="n">
-        <v>236</v>
+        <v>1026</v>
       </c>
       <c r="N15" t="n">
-        <v>298</v>
+        <v>1352</v>
       </c>
       <c r="O15" t="n">
-        <v>369</v>
+        <v>1329</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>0.43906</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.177209</v>
+        <v>0.561616</v>
       </c>
       <c r="R15" t="n">
-        <v>0.245831</v>
+        <v>0.420777</v>
       </c>
       <c r="S15" t="n">
-        <v>0.76434</v>
+        <v>0.604287</v>
       </c>
       <c r="T15" t="n">
-        <v>0.311437</v>
+        <v>0.5342519999999999</v>
       </c>
       <c r="U15" t="n">
-        <v>0.662768</v>
+        <v>0.576542</v>
       </c>
       <c r="V15" t="n">
-        <v>0.173736</v>
+        <v>0.429629</v>
       </c>
       <c r="W15" t="n">
-        <v>0.314882</v>
+        <v>0.476789</v>
       </c>
       <c r="X15" t="n">
-        <v>1.364153</v>
+        <v>0.489959</v>
       </c>
       <c r="Y15" t="n">
-        <v>1.903592</v>
+        <v>1.421805</v>
       </c>
       <c r="Z15" t="n">
-        <v>1.465834</v>
+        <v>1.176143</v>
       </c>
       <c r="AA15" t="n">
-        <v>1.531231</v>
+        <v>1.448214</v>
       </c>
       <c r="AB15" t="n">
-        <v>2.10455</v>
+        <v>1.496248</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.8476590000000001</v>
+        <v>0.775025</v>
       </c>
       <c r="AD15" t="n">
-        <v>0.407622</v>
+        <v>1.468103</v>
       </c>
       <c r="AE15" t="n">
-        <v>47.011952</v>
+        <v>23.169601</v>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ATIVIDADES PROFISSIONAIS, CIENTÍFICAS E TÉCNICAS</t>
+          <t>ATIVIDADES IMOBILIÁRIAS</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>156</v>
+        <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>514</v>
+        <v>13</v>
       </c>
       <c r="F16" t="n">
-        <v>583</v>
+        <v>31</v>
       </c>
       <c r="G16" t="n">
-        <v>671</v>
+        <v>17</v>
       </c>
       <c r="H16" t="n">
-        <v>816</v>
+        <v>76</v>
       </c>
       <c r="I16" t="n">
-        <v>533</v>
+        <v>25</v>
       </c>
       <c r="J16" t="n">
-        <v>683</v>
+        <v>40</v>
       </c>
       <c r="K16" t="n">
-        <v>625</v>
+        <v>180</v>
       </c>
       <c r="L16" t="n">
-        <v>772</v>
+        <v>251</v>
       </c>
       <c r="M16" t="n">
-        <v>1151</v>
+        <v>236</v>
       </c>
       <c r="N16" t="n">
-        <v>1541</v>
+        <v>298</v>
       </c>
       <c r="O16" t="n">
-        <v>1683</v>
+        <v>369</v>
       </c>
       <c r="P16" t="n">
-        <v>0.526645</v>
+        <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.414522</v>
+        <v>0.177209</v>
       </c>
       <c r="R16" t="n">
-        <v>1.052435</v>
+        <v>0.245831</v>
       </c>
       <c r="S16" t="n">
-        <v>0.88961</v>
+        <v>0.76434</v>
       </c>
       <c r="T16" t="n">
-        <v>0.9451889999999999</v>
+        <v>0.311437</v>
       </c>
       <c r="U16" t="n">
-        <v>0.9531539999999999</v>
+        <v>0.662768</v>
       </c>
       <c r="V16" t="n">
-        <v>0.589715</v>
+        <v>0.173736</v>
       </c>
       <c r="W16" t="n">
-        <v>0.720955</v>
+        <v>0.314882</v>
       </c>
       <c r="X16" t="n">
-        <v>0.632736</v>
+        <v>1.364153</v>
       </c>
       <c r="Y16" t="n">
-        <v>0.697417</v>
+        <v>1.903592</v>
       </c>
       <c r="Z16" t="n">
-        <v>0.8539099999999999</v>
+        <v>1.465834</v>
       </c>
       <c r="AA16" t="n">
-        <v>0.862697</v>
+        <v>1.531231</v>
       </c>
       <c r="AB16" t="n">
-        <v>0.873132</v>
+        <v>2.10455</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.770163</v>
+        <v>0.8476590000000001</v>
       </c>
       <c r="AD16" t="n">
-        <v>1.859155</v>
+        <v>0.407622</v>
       </c>
       <c r="AE16" t="n">
-        <v>118.005181</v>
+        <v>47.011952</v>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
@@ -1994,100 +1890,100 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>M</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ATIVIDADES ADMINISTRATIVAS E SERVIÇOS COMPLEMENTARES</t>
+          <t>ATIVIDADES PROFISSIONAIS, CIENTÍFICAS E TÉCNICAS</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1040</v>
+        <v>161</v>
       </c>
       <c r="D17" t="n">
-        <v>3855</v>
+        <v>156</v>
       </c>
       <c r="E17" t="n">
-        <v>4655</v>
+        <v>514</v>
       </c>
       <c r="F17" t="n">
-        <v>4454</v>
+        <v>583</v>
       </c>
       <c r="G17" t="n">
-        <v>3154</v>
+        <v>671</v>
       </c>
       <c r="H17" t="n">
-        <v>3835</v>
+        <v>816</v>
       </c>
       <c r="I17" t="n">
-        <v>5791</v>
+        <v>533</v>
       </c>
       <c r="J17" t="n">
-        <v>6030</v>
+        <v>683</v>
       </c>
       <c r="K17" t="n">
-        <v>4824</v>
+        <v>625</v>
       </c>
       <c r="L17" t="n">
-        <v>7942</v>
+        <v>772</v>
       </c>
       <c r="M17" t="n">
-        <v>9104</v>
+        <v>1151</v>
       </c>
       <c r="N17" t="n">
-        <v>9786</v>
+        <v>1541</v>
       </c>
       <c r="O17" t="n">
-        <v>11443</v>
+        <v>1683</v>
       </c>
       <c r="P17" t="n">
-        <v>0.635027</v>
+        <v>0.526645</v>
       </c>
       <c r="Q17" t="n">
-        <v>1.942517</v>
+        <v>0.414522</v>
       </c>
       <c r="R17" t="n">
-        <v>1.797355</v>
+        <v>1.052435</v>
       </c>
       <c r="S17" t="n">
-        <v>1.676638</v>
+        <v>0.88961</v>
       </c>
       <c r="T17" t="n">
-        <v>1.176997</v>
+        <v>0.9451889999999999</v>
       </c>
       <c r="U17" t="n">
-        <v>1.03618</v>
+        <v>0.9531539999999999</v>
       </c>
       <c r="V17" t="n">
-        <v>1.609196</v>
+        <v>0.589715</v>
       </c>
       <c r="W17" t="n">
-        <v>1.620769</v>
+        <v>0.720955</v>
       </c>
       <c r="X17" t="n">
-        <v>1.250604</v>
+        <v>0.632736</v>
       </c>
       <c r="Y17" t="n">
-        <v>1.744676</v>
+        <v>0.697417</v>
       </c>
       <c r="Z17" t="n">
-        <v>1.766218</v>
+        <v>0.8539099999999999</v>
       </c>
       <c r="AA17" t="n">
-        <v>1.498551</v>
+        <v>0.862697</v>
       </c>
       <c r="AB17" t="n">
-        <v>1.553833</v>
+        <v>0.873132</v>
       </c>
       <c r="AC17" t="n">
-        <v>1.485274</v>
+        <v>0.770163</v>
       </c>
       <c r="AD17" t="n">
-        <v>12.640707</v>
+        <v>1.859155</v>
       </c>
       <c r="AE17" t="n">
-        <v>44.082095</v>
+        <v>118.005181</v>
       </c>
       <c r="AF17" t="inlineStr">
         <is>
@@ -2098,730 +1994,834 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>O</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ADMINISTRAÇÃO PÚBLICA, DEFESA E SEGURIDADE SOCIAL</t>
+          <t>ATIVIDADES ADMINISTRATIVAS E SERVIÇOS COMPLEMENTARES</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3391</v>
+        <v>1040</v>
       </c>
       <c r="D18" t="n">
-        <v>3382</v>
+        <v>3855</v>
       </c>
       <c r="E18" t="n">
-        <v>6299</v>
+        <v>4655</v>
       </c>
       <c r="F18" t="n">
-        <v>4457</v>
+        <v>4454</v>
       </c>
       <c r="G18" t="n">
-        <v>7530</v>
+        <v>3154</v>
       </c>
       <c r="H18" t="n">
-        <v>9138</v>
+        <v>3835</v>
       </c>
       <c r="I18" t="n">
-        <v>10318</v>
+        <v>5791</v>
       </c>
       <c r="J18" t="n">
-        <v>10905</v>
+        <v>6030</v>
       </c>
       <c r="K18" t="n">
-        <v>9869</v>
+        <v>4824</v>
       </c>
       <c r="L18" t="n">
-        <v>5498</v>
+        <v>7942</v>
       </c>
       <c r="M18" t="n">
-        <v>5078</v>
+        <v>9104</v>
       </c>
       <c r="N18" t="n">
-        <v>6107</v>
+        <v>9786</v>
       </c>
       <c r="O18" t="n">
-        <v>7211</v>
+        <v>11443</v>
       </c>
       <c r="P18" t="n">
-        <v>0.336965</v>
+        <v>0.635027</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.248492</v>
+        <v>1.942517</v>
       </c>
       <c r="R18" t="n">
-        <v>0.372944</v>
+        <v>1.797355</v>
       </c>
       <c r="S18" t="n">
-        <v>0.275832</v>
+        <v>1.676638</v>
       </c>
       <c r="T18" t="n">
-        <v>0.387277</v>
+        <v>1.176997</v>
       </c>
       <c r="U18" t="n">
-        <v>0.414734</v>
+        <v>1.03618</v>
       </c>
       <c r="V18" t="n">
-        <v>0.488773</v>
+        <v>1.609196</v>
       </c>
       <c r="W18" t="n">
-        <v>0.490374</v>
+        <v>1.620769</v>
       </c>
       <c r="X18" t="n">
-        <v>0.44233</v>
+        <v>1.250604</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.22935</v>
+        <v>1.744676</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.210675</v>
+        <v>1.766218</v>
       </c>
       <c r="AA18" t="n">
-        <v>0.237252</v>
+        <v>1.498551</v>
       </c>
       <c r="AB18" t="n">
-        <v>0.232131</v>
+        <v>1.553833</v>
       </c>
       <c r="AC18" t="n">
-        <v>0.335933</v>
+        <v>1.485274</v>
       </c>
       <c r="AD18" t="n">
-        <v>7.965755</v>
+        <v>12.640707</v>
       </c>
       <c r="AE18" t="n">
-        <v>31.156784</v>
+        <v>44.082095</v>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>7/12</t>
+          <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>O</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EDUCAÇÃO</t>
+          <t>ADMINISTRAÇÃO PÚBLICA, DEFESA E SEGURIDADE SOCIAL</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>3391</v>
       </c>
       <c r="D19" t="n">
-        <v>876</v>
+        <v>3382</v>
       </c>
       <c r="E19" t="n">
-        <v>1051</v>
+        <v>6299</v>
       </c>
       <c r="F19" t="n">
-        <v>1322</v>
+        <v>4457</v>
       </c>
       <c r="G19" t="n">
-        <v>1513</v>
+        <v>7530</v>
       </c>
       <c r="H19" t="n">
-        <v>1838</v>
+        <v>9138</v>
       </c>
       <c r="I19" t="n">
-        <v>1996</v>
+        <v>10318</v>
       </c>
       <c r="J19" t="n">
-        <v>2265</v>
+        <v>10905</v>
       </c>
       <c r="K19" t="n">
-        <v>2588</v>
+        <v>9869</v>
       </c>
       <c r="L19" t="n">
-        <v>6932</v>
+        <v>5498</v>
       </c>
       <c r="M19" t="n">
-        <v>6229</v>
+        <v>5078</v>
       </c>
       <c r="N19" t="n">
-        <v>9650</v>
+        <v>6107</v>
       </c>
       <c r="O19" t="n">
-        <v>12833</v>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>7211</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.336965</v>
       </c>
       <c r="Q19" t="n">
-        <v>1.093448</v>
+        <v>0.248492</v>
       </c>
       <c r="R19" t="n">
-        <v>1.06935</v>
+        <v>0.372944</v>
       </c>
       <c r="S19" t="n">
-        <v>0.906619</v>
+        <v>0.275832</v>
       </c>
       <c r="T19" t="n">
-        <v>1.222242</v>
+        <v>0.387277</v>
       </c>
       <c r="U19" t="n">
-        <v>1.08893</v>
+        <v>0.414734</v>
       </c>
       <c r="V19" t="n">
-        <v>1.027401</v>
+        <v>0.488773</v>
       </c>
       <c r="W19" t="n">
-        <v>0.91742</v>
+        <v>0.490374</v>
       </c>
       <c r="X19" t="n">
-        <v>0.955286</v>
+        <v>0.44233</v>
       </c>
       <c r="Y19" t="n">
-        <v>2.524554</v>
+        <v>0.22935</v>
       </c>
       <c r="Z19" t="n">
-        <v>2.630518</v>
+        <v>0.210675</v>
       </c>
       <c r="AA19" t="n">
-        <v>1.782708</v>
+        <v>0.237252</v>
       </c>
       <c r="AB19" t="n">
-        <v>2.516928</v>
+        <v>0.232131</v>
       </c>
       <c r="AC19" t="n">
-        <v>1.47795</v>
+        <v>0.335933</v>
       </c>
       <c r="AD19" t="n">
-        <v>14.176194</v>
+        <v>7.965755</v>
       </c>
       <c r="AE19" t="n">
-        <v>85.126947</v>
+        <v>31.156784</v>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>11/12</t>
+          <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SAÚDE HUMANA E SERVIÇOS SOCIAIS</t>
+          <t>EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>576</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>571</v>
+        <v>876</v>
       </c>
       <c r="E20" t="n">
-        <v>637</v>
+        <v>1051</v>
       </c>
       <c r="F20" t="n">
-        <v>1834</v>
+        <v>1322</v>
       </c>
       <c r="G20" t="n">
-        <v>1957</v>
+        <v>1513</v>
       </c>
       <c r="H20" t="n">
-        <v>2083</v>
+        <v>1838</v>
       </c>
       <c r="I20" t="n">
-        <v>2073</v>
+        <v>1996</v>
       </c>
       <c r="J20" t="n">
-        <v>2515</v>
+        <v>2265</v>
       </c>
       <c r="K20" t="n">
-        <v>2777</v>
+        <v>2588</v>
       </c>
       <c r="L20" t="n">
-        <v>3172</v>
+        <v>6932</v>
       </c>
       <c r="M20" t="n">
-        <v>3658</v>
+        <v>6229</v>
       </c>
       <c r="N20" t="n">
-        <v>3202</v>
+        <v>9650</v>
       </c>
       <c r="O20" t="n">
-        <v>3327</v>
-      </c>
-      <c r="P20" t="n">
-        <v>0.608935</v>
+        <v>12833</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="Q20" t="n">
-        <v>0.555183</v>
+        <v>1.093448</v>
       </c>
       <c r="R20" t="n">
-        <v>0.538399</v>
+        <v>1.06935</v>
       </c>
       <c r="S20" t="n">
-        <v>1.469437</v>
+        <v>0.906619</v>
       </c>
       <c r="T20" t="n">
-        <v>1.489968</v>
+        <v>1.222242</v>
       </c>
       <c r="U20" t="n">
-        <v>1.353741</v>
+        <v>1.08893</v>
       </c>
       <c r="V20" t="n">
-        <v>1.194519</v>
+        <v>1.027401</v>
       </c>
       <c r="W20" t="n">
-        <v>1.133038</v>
+        <v>0.91742</v>
       </c>
       <c r="X20" t="n">
-        <v>1.09314</v>
+        <v>0.955286</v>
       </c>
       <c r="Y20" t="n">
-        <v>1.371292</v>
+        <v>2.524554</v>
       </c>
       <c r="Z20" t="n">
-        <v>1.33919</v>
+        <v>2.630518</v>
       </c>
       <c r="AA20" t="n">
-        <v>0.900875</v>
+        <v>1.782708</v>
       </c>
       <c r="AB20" t="n">
-        <v>0.853013</v>
+        <v>2.516928</v>
       </c>
       <c r="AC20" t="n">
-        <v>1.069287</v>
+        <v>1.47795</v>
       </c>
       <c r="AD20" t="n">
-        <v>3.675228</v>
+        <v>14.176194</v>
       </c>
       <c r="AE20" t="n">
-        <v>4.886507</v>
+        <v>85.126947</v>
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>11/12</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ARTES, CULTURA, ESPORTE E RECREAÇÃO</t>
+          <t>SAÚDE HUMANA E SERVIÇOS SOCIAIS</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>86</v>
+        <v>576</v>
       </c>
       <c r="D21" t="n">
-        <v>115</v>
+        <v>571</v>
       </c>
       <c r="E21" t="n">
-        <v>93</v>
+        <v>637</v>
       </c>
       <c r="F21" t="n">
-        <v>131</v>
+        <v>1834</v>
       </c>
       <c r="G21" t="n">
-        <v>141</v>
+        <v>1957</v>
       </c>
       <c r="H21" t="n">
-        <v>207</v>
+        <v>2083</v>
       </c>
       <c r="I21" t="n">
-        <v>213</v>
+        <v>2073</v>
       </c>
       <c r="J21" t="n">
-        <v>256</v>
+        <v>2515</v>
       </c>
       <c r="K21" t="n">
-        <v>260</v>
+        <v>2777</v>
       </c>
       <c r="L21" t="n">
-        <v>290</v>
+        <v>3172</v>
       </c>
       <c r="M21" t="n">
-        <v>350</v>
+        <v>3658</v>
       </c>
       <c r="N21" t="n">
-        <v>445</v>
+        <v>3202</v>
       </c>
       <c r="O21" t="n">
-        <v>575</v>
+        <v>3327</v>
       </c>
       <c r="P21" t="n">
-        <v>0.567574</v>
+        <v>0.608935</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.696394</v>
+        <v>0.555183</v>
       </c>
       <c r="R21" t="n">
-        <v>0.510064</v>
+        <v>0.538399</v>
       </c>
       <c r="S21" t="n">
-        <v>0.6834519999999999</v>
+        <v>1.469437</v>
       </c>
       <c r="T21" t="n">
-        <v>0.721378</v>
+        <v>1.489968</v>
       </c>
       <c r="U21" t="n">
-        <v>0.881933</v>
+        <v>1.353741</v>
       </c>
       <c r="V21" t="n">
-        <v>0.983508</v>
+        <v>1.194519</v>
       </c>
       <c r="W21" t="n">
-        <v>0.8218800000000001</v>
+        <v>1.133038</v>
       </c>
       <c r="X21" t="n">
-        <v>0.857727</v>
+        <v>1.09314</v>
       </c>
       <c r="Y21" t="n">
-        <v>1.277689</v>
+        <v>1.371292</v>
       </c>
       <c r="Z21" t="n">
-        <v>1.61837</v>
+        <v>1.33919</v>
       </c>
       <c r="AA21" t="n">
-        <v>1.362921</v>
+        <v>0.900875</v>
       </c>
       <c r="AB21" t="n">
-        <v>1.419695</v>
+        <v>0.853013</v>
       </c>
       <c r="AC21" t="n">
-        <v>0.954045</v>
+        <v>1.069287</v>
       </c>
       <c r="AD21" t="n">
-        <v>0.635184</v>
+        <v>3.675228</v>
       </c>
       <c r="AE21" t="n">
-        <v>98.275862</v>
+        <v>4.886507</v>
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>11/12</t>
+          <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>OUTRAS ATIVIDADES DE SERVIÇOS</t>
+          <t>ARTES, CULTURA, ESPORTE E RECREAÇÃO</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>609</v>
+        <v>86</v>
       </c>
       <c r="D22" t="n">
-        <v>675</v>
+        <v>115</v>
       </c>
       <c r="E22" t="n">
-        <v>756</v>
+        <v>93</v>
       </c>
       <c r="F22" t="n">
-        <v>518</v>
+        <v>131</v>
       </c>
       <c r="G22" t="n">
-        <v>544</v>
+        <v>141</v>
       </c>
       <c r="H22" t="n">
-        <v>579</v>
+        <v>207</v>
       </c>
       <c r="I22" t="n">
-        <v>627</v>
+        <v>213</v>
       </c>
       <c r="J22" t="n">
-        <v>616</v>
+        <v>256</v>
       </c>
       <c r="K22" t="n">
-        <v>844</v>
+        <v>260</v>
       </c>
       <c r="L22" t="n">
-        <v>895</v>
+        <v>290</v>
       </c>
       <c r="M22" t="n">
-        <v>1049</v>
+        <v>350</v>
       </c>
       <c r="N22" t="n">
-        <v>849</v>
+        <v>445</v>
       </c>
       <c r="O22" t="n">
-        <v>1050</v>
+        <v>575</v>
       </c>
       <c r="P22" t="n">
-        <v>0.69369</v>
+        <v>0.567574</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.633938</v>
+        <v>0.696394</v>
       </c>
       <c r="R22" t="n">
-        <v>0.703484</v>
+        <v>0.510064</v>
       </c>
       <c r="S22" t="n">
-        <v>0.498673</v>
+        <v>0.6834519999999999</v>
       </c>
       <c r="T22" t="n">
-        <v>0.5738529999999999</v>
+        <v>0.721378</v>
       </c>
       <c r="U22" t="n">
-        <v>0.557488</v>
+        <v>0.881933</v>
       </c>
       <c r="V22" t="n">
-        <v>0.628477</v>
+        <v>0.983508</v>
       </c>
       <c r="W22" t="n">
-        <v>0.529511</v>
+        <v>0.8218800000000001</v>
       </c>
       <c r="X22" t="n">
-        <v>0.764243</v>
+        <v>0.857727</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.836153</v>
+        <v>1.277689</v>
       </c>
       <c r="Z22" t="n">
-        <v>0.964286</v>
+        <v>1.61837</v>
       </c>
       <c r="AA22" t="n">
-        <v>0.5978250000000001</v>
+        <v>1.362921</v>
       </c>
       <c r="AB22" t="n">
-        <v>0.735486</v>
+        <v>1.419695</v>
       </c>
       <c r="AC22" t="n">
-        <v>0.670547</v>
+        <v>0.954045</v>
       </c>
       <c r="AD22" t="n">
-        <v>1.159901</v>
+        <v>0.635184</v>
       </c>
       <c r="AE22" t="n">
-        <v>17.318436</v>
+        <v>98.275862</v>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>11/12</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>S</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SERVIÇOS DOMÉSTICOS</t>
+          <t>OUTRAS ATIVIDADES DE SERVIÇOS</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>609</v>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>675</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>756</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>518</v>
       </c>
       <c r="G23" t="n">
-        <v>8</v>
+        <v>544</v>
       </c>
       <c r="H23" t="n">
-        <v>7</v>
+        <v>579</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>627</v>
       </c>
       <c r="J23" t="n">
-        <v>7</v>
+        <v>616</v>
       </c>
       <c r="K23" t="n">
-        <v>10</v>
+        <v>844</v>
       </c>
       <c r="L23" t="n">
-        <v>10</v>
+        <v>895</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>1049</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>849</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>1050</v>
       </c>
       <c r="P23" t="n">
-        <v>0.655625</v>
+        <v>0.69369</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.386525</v>
+        <v>0.633938</v>
       </c>
       <c r="R23" t="n">
-        <v>0.275496</v>
+        <v>0.703484</v>
       </c>
       <c r="S23" t="n">
-        <v>0.48443</v>
+        <v>0.498673</v>
       </c>
       <c r="T23" t="n">
-        <v>0.702868</v>
+        <v>0.5738529999999999</v>
       </c>
       <c r="U23" t="n">
-        <v>0.666344</v>
+        <v>0.557488</v>
       </c>
       <c r="V23" t="n">
-        <v>0</v>
+        <v>0.628477</v>
       </c>
       <c r="W23" t="n">
-        <v>1.434728</v>
+        <v>0.529511</v>
       </c>
       <c r="X23" t="n">
-        <v>2.656186</v>
+        <v>0.764243</v>
       </c>
       <c r="Y23" t="n">
-        <v>2.50273</v>
+        <v>0.836153</v>
       </c>
       <c r="Z23" t="n">
-        <v>0</v>
+        <v>0.964286</v>
       </c>
       <c r="AA23" t="n">
-        <v>0</v>
+        <v>0.5978250000000001</v>
       </c>
       <c r="AB23" t="n">
-        <v>0</v>
+        <v>0.735486</v>
       </c>
       <c r="AC23" t="n">
-        <v>0.751149</v>
+        <v>0.670547</v>
       </c>
       <c r="AD23" t="n">
-        <v>0</v>
+        <v>1.159901</v>
       </c>
       <c r="AE23" t="n">
-        <v>-100</v>
+        <v>17.318436</v>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>4/12</t>
+          <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SERVIÇOS DOMÉSTICOS</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>8</v>
+      </c>
+      <c r="H24" t="n">
+        <v>7</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7</v>
+      </c>
+      <c r="K24" t="n">
+        <v>10</v>
+      </c>
+      <c r="L24" t="n">
+        <v>10</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.655625</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.386525</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.275496</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.48443</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.702868</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0.666344</v>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" t="n">
+        <v>1.434728</v>
+      </c>
+      <c r="X24" t="n">
+        <v>2.656186</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>2.50273</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0.751149</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>-100</v>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>4/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>U</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>ORGANISMOS INTERNACIONAIS E OUTRAS INSTITUIÇÕES EXTRATERRITORIAIS</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C25" t="n">
         <v>5</v>
       </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="n">
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
         <v>12.331998</v>
       </c>
-      <c r="Q24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC24" t="n">
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="n">
         <v>0.948615</v>
       </c>
-      <c r="AD24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE24" t="inlineStr">
+      <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AF24" t="inlineStr">
+      <c r="AF25" t="inlineStr">
         <is>
           <t>0/12</t>
         </is>

</xml_diff>

<commit_message>
Aplica formatação visual (mesma paleta da referência) nas planilhas de Ananindeua/Capanema
Título azul #1E2A5E em negrito, nota em cinza, cabeçalho branco em negrito
com fundo azul, linhas de dados zebradas (F4F4F4/FFFFFF), congelamento de
painel na primeira linha de dados — replica exatamente o estilo visual
usado nos arquivos de Imperatriz (prjeto_vetor_municipal/planilhas/),
que eu tinha deixado sem nenhuma formatação (só preto e branco).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Empregos_por_Secao_CNAE_RAIS_Ananindeua.xlsx
+++ b/Empregos_por_Secao_CNAE_RAIS_Ananindeua.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,13 +32,47 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001E2A5E"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E2A5E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F4F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -53,10 +87,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,2409 +468,2414 @@
   <dimension ref="A1:AF25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="14" customWidth="1" min="29" max="29"/>
-    <col width="14" customWidth="1" min="30" max="30"/>
-    <col width="14" customWidth="1" min="31" max="31"/>
-    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>EMPREGOS POR SEÇÃO CNAE (RAIS) — ANANINDEUA vs PARÁ — SÉRIE 2001-2025</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Vínculos empregatícios ativos em 31/12. QL calculado no nível de Seção. Fonte: RAIS/MTE.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Seção</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Nome Seção</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2001</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2003</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2005</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2007</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2009</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2011</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2013</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2015</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2017</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2019</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2021</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2023</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Emp. 2025</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>QL 2001</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>QL 2003</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>QL 2005</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr">
+      <c r="S4" s="5" t="inlineStr">
         <is>
           <t>QL 2007</t>
         </is>
       </c>
-      <c r="T4" s="2" t="inlineStr">
+      <c r="T4" s="5" t="inlineStr">
         <is>
           <t>QL 2009</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr">
+      <c r="U4" s="5" t="inlineStr">
         <is>
           <t>QL 2011</t>
         </is>
       </c>
-      <c r="V4" s="2" t="inlineStr">
+      <c r="V4" s="5" t="inlineStr">
         <is>
           <t>QL 2013</t>
         </is>
       </c>
-      <c r="W4" s="2" t="inlineStr">
+      <c r="W4" s="5" t="inlineStr">
         <is>
           <t>QL 2015</t>
         </is>
       </c>
-      <c r="X4" s="2" t="inlineStr">
+      <c r="X4" s="5" t="inlineStr">
         <is>
           <t>QL 2017</t>
         </is>
       </c>
-      <c r="Y4" s="2" t="inlineStr">
+      <c r="Y4" s="5" t="inlineStr">
         <is>
           <t>QL 2019</t>
         </is>
       </c>
-      <c r="Z4" s="2" t="inlineStr">
+      <c r="Z4" s="5" t="inlineStr">
         <is>
           <t>QL 2021</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
+      <c r="AA4" s="5" t="inlineStr">
         <is>
           <t>QL 2023</t>
         </is>
       </c>
-      <c r="AB4" s="2" t="inlineStr">
+      <c r="AB4" s="5" t="inlineStr">
         <is>
           <t>QL 2025</t>
         </is>
       </c>
-      <c r="AC4" s="2" t="inlineStr">
+      <c r="AC4" s="5" t="inlineStr">
         <is>
           <t>QL Médio</t>
         </is>
       </c>
-      <c r="AD4" s="2" t="inlineStr">
+      <c r="AD4" s="5" t="inlineStr">
         <is>
           <t>Representat. (%)</t>
         </is>
       </c>
-      <c r="AE4" s="2" t="inlineStr">
+      <c r="AE4" s="5" t="inlineStr">
         <is>
           <t>Cresc. 5 anos (%)</t>
         </is>
       </c>
-      <c r="AF4" s="2" t="inlineStr">
+      <c r="AF4" s="5" t="inlineStr">
         <is>
           <t>Consistência (0-12)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>AGRICULTURA, PECUÁRIA, PRODUÇÃO FLORESTAL, PESCA E AQÜICULTURA</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="7" t="n">
         <v>200</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="7" t="n">
         <v>136</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="7" t="n">
         <v>102</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="7" t="n">
         <v>1876</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="7" t="n">
         <v>1506</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="7" t="n">
         <v>1522</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="7" t="n">
         <v>1334</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="7" t="n">
         <v>1715</v>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="7" t="n">
         <v>1990</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="7" t="n">
         <v>2144</v>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" s="7" t="n">
         <v>2286</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N5" s="7" t="n">
         <v>181</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5" s="7" t="n">
         <v>190</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="7" t="n">
         <v>0.219934</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q5" s="7" t="n">
         <v>0.087952</v>
       </c>
-      <c r="R5" t="n">
+      <c r="R5" s="7" t="n">
         <v>0.047489</v>
       </c>
-      <c r="S5" t="n">
+      <c r="S5" s="7" t="n">
         <v>0.702551</v>
       </c>
-      <c r="T5" t="n">
+      <c r="T5" s="7" t="n">
         <v>0.630103</v>
       </c>
-      <c r="U5" t="n">
+      <c r="U5" s="7" t="n">
         <v>0.521001</v>
       </c>
-      <c r="V5" t="n">
+      <c r="V5" s="7" t="n">
         <v>0.445373</v>
       </c>
-      <c r="W5" t="n">
+      <c r="W5" s="7" t="n">
         <v>0.541066</v>
       </c>
-      <c r="X5" t="n">
+      <c r="X5" s="7" t="n">
         <v>0.6203650000000001</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Y5" s="7" t="n">
         <v>0.889655</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="Z5" s="7" t="n">
         <v>0.864854</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AA5" s="7" t="n">
         <v>0.058522</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AB5" s="7" t="n">
         <v>0.065429</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AC5" s="7" t="n">
         <v>0.438023</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AD5" s="7" t="n">
         <v>0.209887</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AE5" s="7" t="n">
         <v>-91.13806</v>
       </c>
-      <c r="AF5" t="inlineStr">
+      <c r="AF5" s="7" t="inlineStr">
         <is>
           <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>INDÚSTRIAS EXTRATIVAS</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="9" t="n">
         <v>96</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="9" t="n">
         <v>85</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="9" t="n">
         <v>59</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="9" t="n">
         <v>160</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="9" t="n">
         <v>120</v>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="9" t="n">
         <v>99</v>
       </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
+      <c r="L6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" s="9" t="n">
         <v>37</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6" s="9" t="n">
         <v>0.569169</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q6" s="9" t="n">
         <v>0.323031</v>
       </c>
-      <c r="R6" t="n">
+      <c r="R6" s="9" t="n">
         <v>0.157789</v>
       </c>
-      <c r="S6" t="n">
+      <c r="S6" s="9" t="n">
         <v>0.262257</v>
       </c>
-      <c r="T6" t="n">
+      <c r="T6" s="9" t="n">
         <v>0.180862</v>
       </c>
-      <c r="U6" t="n">
+      <c r="U6" s="9" t="n">
         <v>0.108343</v>
       </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0</v>
-      </c>
-      <c r="X6" t="n">
+      <c r="V6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="9" t="n">
         <v>0.003342</v>
       </c>
-      <c r="Y6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" t="n">
+      <c r="Y6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="9" t="n">
         <v>0.002574</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AB6" s="9" t="n">
         <v>0.045367</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AC6" s="9" t="n">
         <v>0.127133</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AD6" s="9" t="n">
         <v>0.040873</v>
       </c>
-      <c r="AE6" t="inlineStr">
+      <c r="AE6" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AF6" t="inlineStr">
+      <c r="AF6" s="9" t="inlineStr">
         <is>
           <t>4/12</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>INDÚSTRIAS DE TRANSFORMAÇÃO</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="7" t="n">
         <v>6174</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="7" t="n">
         <v>7517</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="7" t="n">
         <v>8592</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="7" t="n">
         <v>5535</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="7" t="n">
         <v>4902</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="7" t="n">
         <v>5454</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="7" t="n">
         <v>5291</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" s="7" t="n">
         <v>5383</v>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="7" t="n">
         <v>5330</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="7" t="n">
         <v>5946</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="7" t="n">
         <v>6521</v>
       </c>
-      <c r="N7" t="n">
+      <c r="N7" s="7" t="n">
         <v>8729</v>
       </c>
-      <c r="O7" t="n">
+      <c r="O7" s="7" t="n">
         <v>9889</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P7" s="7" t="n">
         <v>1.87852</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q7" s="7" t="n">
         <v>1.665559</v>
       </c>
-      <c r="R7" t="n">
+      <c r="R7" s="7" t="n">
         <v>1.470426</v>
       </c>
-      <c r="S7" t="n">
+      <c r="S7" s="7" t="n">
         <v>1.329939</v>
       </c>
-      <c r="T7" t="n">
+      <c r="T7" s="7" t="n">
         <v>1.298055</v>
       </c>
-      <c r="U7" t="n">
+      <c r="U7" s="7" t="n">
         <v>1.366357</v>
       </c>
-      <c r="V7" t="n">
+      <c r="V7" s="7" t="n">
         <v>1.347573</v>
       </c>
-      <c r="W7" t="n">
+      <c r="W7" s="7" t="n">
         <v>1.269484</v>
       </c>
-      <c r="X7" t="n">
+      <c r="X7" s="7" t="n">
         <v>1.272711</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Y7" s="7" t="n">
         <v>1.043302</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="Z7" s="7" t="n">
         <v>1.013227</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AA7" s="7" t="n">
         <v>1.238425</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AB7" s="7" t="n">
         <v>1.298093</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AC7" s="7" t="n">
         <v>1.345513</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AD7" s="7" t="n">
         <v>10.924054</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AE7" s="7" t="n">
         <v>66.31348800000001</v>
       </c>
-      <c r="AF7" t="inlineStr">
+      <c r="AF7" s="7" t="inlineStr">
         <is>
           <t>8/12</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>ELETRICIDADE E GÁS</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="C8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="9" t="n">
         <v>142</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" s="9" t="n">
         <v>152</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="n">
+      <c r="L8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="9" t="n">
         <v>0.042232</v>
       </c>
-      <c r="R8" t="n">
+      <c r="R8" s="9" t="n">
         <v>0.028148</v>
       </c>
-      <c r="S8" t="n">
+      <c r="S8" s="9" t="n">
         <v>0.836732</v>
       </c>
-      <c r="T8" t="n">
+      <c r="T8" s="9" t="n">
         <v>1.140237</v>
       </c>
-      <c r="U8" t="n">
+      <c r="U8" s="9" t="n">
         <v>0.145961</v>
       </c>
-      <c r="V8" t="n">
+      <c r="V8" s="9" t="n">
         <v>0.006051</v>
       </c>
-      <c r="W8" t="n">
+      <c r="W8" s="9" t="n">
         <v>0.076768</v>
       </c>
-      <c r="X8" t="n">
+      <c r="X8" s="9" t="n">
         <v>0.087432</v>
       </c>
-      <c r="Y8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC8" t="n">
+      <c r="Y8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="9" t="n">
         <v>0.181812</v>
       </c>
-      <c r="AD8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE8" t="inlineStr">
+      <c r="AD8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AF8" t="inlineStr">
+      <c r="AF8" s="9" t="inlineStr">
         <is>
           <t>4/12</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>ÁGUA, ESGOTO, ATIVIDADES DE GESTÃO DE RESÍDUOS E DESCONTAMINAÇÃO</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="7" t="n">
         <v>37</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="7" t="n">
         <v>128</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="7" t="n">
         <v>202</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="7" t="n">
         <v>124</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" s="7" t="n">
         <v>249</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="7" t="n">
         <v>126</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="7" t="n">
         <v>325</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="7" t="n">
         <v>446</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="7" t="n">
         <v>563</v>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" s="7" t="n">
         <v>583</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N9" s="7" t="n">
         <v>1555</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O9" s="7" t="n">
         <v>1460</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9" s="7" t="n">
         <v>0.238892</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q9" s="7" t="n">
         <v>0.649322</v>
       </c>
-      <c r="R9" t="n">
+      <c r="R9" s="7" t="n">
         <v>1.418067</v>
       </c>
-      <c r="S9" t="n">
+      <c r="S9" s="7" t="n">
         <v>0.472557</v>
       </c>
-      <c r="T9" t="n">
+      <c r="T9" s="7" t="n">
         <v>0.708214</v>
       </c>
-      <c r="U9" t="n">
+      <c r="U9" s="7" t="n">
         <v>0.476449</v>
       </c>
-      <c r="V9" t="n">
+      <c r="V9" s="7" t="n">
         <v>1.082969</v>
       </c>
-      <c r="W9" t="n">
+      <c r="W9" s="7" t="n">
         <v>0.917736</v>
       </c>
-      <c r="X9" t="n">
+      <c r="X9" s="7" t="n">
         <v>1.328189</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Y9" s="7" t="n">
         <v>1.463911</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="Z9" s="7" t="n">
         <v>1.311045</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AA9" s="7" t="n">
         <v>3.101239</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AB9" s="7" t="n">
         <v>2.635</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AC9" s="7" t="n">
         <v>1.215661</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AD9" s="7" t="n">
         <v>1.612814</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AE9" s="7" t="n">
         <v>159.325044</v>
       </c>
-      <c r="AF9" t="inlineStr">
+      <c r="AF9" s="7" t="inlineStr">
         <is>
           <t>8/12</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>CONSTRUÇÃO</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="9" t="n">
         <v>2056</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="9" t="n">
         <v>2163</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="9" t="n">
         <v>2795</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="9" t="n">
         <v>4621</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="9" t="n">
         <v>5775</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="9" t="n">
         <v>7692</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="9" t="n">
         <v>6616</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" s="9" t="n">
         <v>7046</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="9" t="n">
         <v>7388</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="9" t="n">
         <v>5530</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" s="9" t="n">
         <v>4956</v>
       </c>
-      <c r="N10" t="n">
+      <c r="N10" s="9" t="n">
         <v>6845</v>
       </c>
-      <c r="O10" t="n">
+      <c r="O10" s="9" t="n">
         <v>5365</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P10" s="9" t="n">
         <v>1.274695</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q10" s="9" t="n">
         <v>1.529866</v>
       </c>
-      <c r="R10" t="n">
+      <c r="R10" s="9" t="n">
         <v>1.335262</v>
       </c>
-      <c r="S10" t="n">
+      <c r="S10" s="9" t="n">
         <v>1.520138</v>
       </c>
-      <c r="T10" t="n">
+      <c r="T10" s="9" t="n">
         <v>1.81171</v>
       </c>
-      <c r="U10" t="n">
+      <c r="U10" s="9" t="n">
         <v>1.630957</v>
       </c>
-      <c r="V10" t="n">
+      <c r="V10" s="9" t="n">
         <v>1.083491</v>
       </c>
-      <c r="W10" t="n">
+      <c r="W10" s="9" t="n">
         <v>1.286973</v>
       </c>
-      <c r="X10" t="n">
+      <c r="X10" s="9" t="n">
         <v>2.037857</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Y10" s="9" t="n">
         <v>2.010576</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="Z10" s="9" t="n">
         <v>1.472667</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AA10" s="9" t="n">
         <v>1.664924</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AB10" s="9" t="n">
         <v>1.311461</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AC10" s="9" t="n">
         <v>1.536198</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AD10" s="9" t="n">
         <v>5.92654</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AE10" s="9" t="n">
         <v>-2.983725</v>
       </c>
-      <c r="AF10" t="inlineStr">
+      <c r="AF10" s="9" t="inlineStr">
         <is>
           <t>8/12</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>COMÉRCIO; REPARAÇÃO DE VEÍCULOS AUTOMOTORES E MOTOCICLETAS</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="7" t="n">
         <v>7415</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="7" t="n">
         <v>10376</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="7" t="n">
         <v>13460</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="7" t="n">
         <v>14277</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="7" t="n">
         <v>14786</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="7" t="n">
         <v>17373</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="7" t="n">
         <v>18382</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" s="7" t="n">
         <v>18780</v>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="7" t="n">
         <v>18207</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="7" t="n">
         <v>17599</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="7" t="n">
         <v>20723</v>
       </c>
-      <c r="N11" t="n">
+      <c r="N11" s="7" t="n">
         <v>22298</v>
       </c>
-      <c r="O11" t="n">
+      <c r="O11" s="7" t="n">
         <v>23853</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P11" s="7" t="n">
         <v>1.691867</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q11" s="7" t="n">
         <v>1.736383</v>
       </c>
-      <c r="R11" t="n">
+      <c r="R11" s="7" t="n">
         <v>1.664573</v>
       </c>
-      <c r="S11" t="n">
+      <c r="S11" s="7" t="n">
         <v>1.602888</v>
       </c>
-      <c r="T11" t="n">
+      <c r="T11" s="7" t="n">
         <v>1.632403</v>
       </c>
-      <c r="U11" t="n">
+      <c r="U11" s="7" t="n">
         <v>1.610082</v>
       </c>
-      <c r="V11" t="n">
+      <c r="V11" s="7" t="n">
         <v>1.583657</v>
       </c>
-      <c r="W11" t="n">
+      <c r="W11" s="7" t="n">
         <v>1.485592</v>
       </c>
-      <c r="X11" t="n">
+      <c r="X11" s="7" t="n">
         <v>1.509385</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Y11" s="7" t="n">
         <v>1.407752</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="Z11" s="7" t="n">
         <v>1.511553</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AA11" s="7" t="n">
         <v>1.51523</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AB11" s="7" t="n">
         <v>1.558071</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AC11" s="7" t="n">
         <v>1.577649</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AD11" s="7" t="n">
         <v>26.349627</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AE11" s="7" t="n">
         <v>35.53611</v>
       </c>
-      <c r="AF11" t="inlineStr">
+      <c r="AF11" s="7" t="inlineStr">
         <is>
           <t>10/12</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>TRANSPORTE, ARMAZENAGEM E CORREIO</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="9" t="n">
         <v>4418</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="9" t="n">
         <v>4814</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="9" t="n">
         <v>5331</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="9" t="n">
         <v>5231</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="9" t="n">
         <v>5270</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="9" t="n">
         <v>6493</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="9" t="n">
         <v>6571</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J12" s="9" t="n">
         <v>7691</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="9" t="n">
         <v>6630</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="9" t="n">
         <v>6074</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="9" t="n">
         <v>5855</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N12" s="9" t="n">
         <v>6645</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O12" s="9" t="n">
         <v>6576</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P12" s="9" t="n">
         <v>3.555985</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="Q12" s="9" t="n">
         <v>3.432463</v>
       </c>
-      <c r="R12" t="n">
+      <c r="R12" s="9" t="n">
         <v>3.071248</v>
       </c>
-      <c r="S12" t="n">
+      <c r="S12" s="9" t="n">
         <v>2.716455</v>
       </c>
-      <c r="T12" t="n">
+      <c r="T12" s="9" t="n">
         <v>2.744492</v>
       </c>
-      <c r="U12" t="n">
+      <c r="U12" s="9" t="n">
         <v>2.803307</v>
       </c>
-      <c r="V12" t="n">
+      <c r="V12" s="9" t="n">
         <v>2.836888</v>
       </c>
-      <c r="W12" t="n">
+      <c r="W12" s="9" t="n">
         <v>2.898363</v>
       </c>
-      <c r="X12" t="n">
+      <c r="X12" s="9" t="n">
         <v>2.597792</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="Y12" s="9" t="n">
         <v>2.332161</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="Z12" s="9" t="n">
         <v>2.103383</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AA12" s="9" t="n">
         <v>2.147584</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AB12" s="9" t="n">
         <v>2.010303</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AC12" s="9" t="n">
         <v>2.711571</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AD12" s="9" t="n">
         <v>7.264292</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AE12" s="9" t="n">
         <v>8.264735</v>
       </c>
-      <c r="AF12" t="inlineStr">
+      <c r="AF12" s="9" t="inlineStr">
         <is>
           <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>ALOJAMENTO E ALIMENTAÇÃO</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="7" t="n">
         <v>401</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="7" t="n">
         <v>936</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="7" t="n">
         <v>1093</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="7" t="n">
         <v>1516</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" s="7" t="n">
         <v>1511</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="7" t="n">
         <v>1961</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="7" t="n">
         <v>1322</v>
       </c>
-      <c r="J13" t="n">
+      <c r="J13" s="7" t="n">
         <v>1338</v>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="7" t="n">
         <v>1577</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="7" t="n">
         <v>1620</v>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" s="7" t="n">
         <v>1900</v>
       </c>
-      <c r="N13" t="n">
+      <c r="N13" s="7" t="n">
         <v>2563</v>
       </c>
-      <c r="O13" t="n">
+      <c r="O13" s="7" t="n">
         <v>2767</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P13" s="7" t="n">
         <v>1.049922</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q13" s="7" t="n">
         <v>1.331174</v>
       </c>
-      <c r="R13" t="n">
+      <c r="R13" s="7" t="n">
         <v>1.253481</v>
       </c>
-      <c r="S13" t="n">
+      <c r="S13" s="7" t="n">
         <v>1.420617</v>
       </c>
-      <c r="T13" t="n">
+      <c r="T13" s="7" t="n">
         <v>1.30352</v>
       </c>
-      <c r="U13" t="n">
+      <c r="U13" s="7" t="n">
         <v>1.400883</v>
       </c>
-      <c r="V13" t="n">
+      <c r="V13" s="7" t="n">
         <v>0.856169</v>
       </c>
-      <c r="W13" t="n">
+      <c r="W13" s="7" t="n">
         <v>0.793826</v>
       </c>
-      <c r="X13" t="n">
+      <c r="X13" s="7" t="n">
         <v>1.06089</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Y13" s="7" t="n">
         <v>0.948354</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="Z13" s="7" t="n">
         <v>1.12726</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AA13" s="7" t="n">
         <v>1.182529</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AB13" s="7" t="n">
         <v>1.13324</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AC13" s="7" t="n">
         <v>1.14322</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AD13" s="7" t="n">
         <v>3.056614</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AE13" s="7" t="n">
         <v>70.802469</v>
       </c>
-      <c r="AF13" t="inlineStr">
+      <c r="AF13" s="7" t="inlineStr">
         <is>
           <t>10/12</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>INFORMAÇÃO E COMUNICAÇÃO</t>
         </is>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="9" t="n">
         <v>47</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="9" t="n">
         <v>43</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" s="9" t="n">
         <v>35</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="9" t="n">
         <v>33</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="9" t="n">
         <v>73</v>
       </c>
-      <c r="J14" t="n">
+      <c r="J14" s="9" t="n">
         <v>125</v>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" s="9" t="n">
         <v>223</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="9" t="n">
         <v>259</v>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" s="9" t="n">
         <v>240</v>
       </c>
-      <c r="N14" t="n">
+      <c r="N14" s="9" t="n">
         <v>536</v>
       </c>
-      <c r="O14" t="n">
+      <c r="O14" s="9" t="n">
         <v>568</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P14" s="9" t="n">
         <v>0.046888</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q14" s="9" t="n">
         <v>0.043606</v>
       </c>
-      <c r="R14" t="n">
+      <c r="R14" s="9" t="n">
         <v>0.116161</v>
       </c>
-      <c r="S14" t="n">
+      <c r="S14" s="9" t="n">
         <v>0.118684</v>
       </c>
-      <c r="T14" t="n">
+      <c r="T14" s="9" t="n">
         <v>0.116535</v>
       </c>
-      <c r="U14" t="n">
+      <c r="U14" s="9" t="n">
         <v>0.08903800000000001</v>
       </c>
-      <c r="V14" t="n">
+      <c r="V14" s="9" t="n">
         <v>0.182388</v>
       </c>
-      <c r="W14" t="n">
+      <c r="W14" s="9" t="n">
         <v>0.244342</v>
       </c>
-      <c r="X14" t="n">
+      <c r="X14" s="9" t="n">
         <v>0.365163</v>
       </c>
-      <c r="Y14" t="n">
+      <c r="Y14" s="9" t="n">
         <v>0.396953</v>
       </c>
-      <c r="Z14" t="n">
+      <c r="Z14" s="9" t="n">
         <v>0.325877</v>
       </c>
-      <c r="AA14" t="n">
+      <c r="AA14" s="9" t="n">
         <v>0.611114</v>
       </c>
-      <c r="AB14" t="n">
+      <c r="AB14" s="9" t="n">
         <v>0.594433</v>
       </c>
-      <c r="AC14" t="n">
+      <c r="AC14" s="9" t="n">
         <v>0.250091</v>
       </c>
-      <c r="AD14" t="n">
+      <c r="AD14" s="9" t="n">
         <v>0.627451</v>
       </c>
-      <c r="AE14" t="n">
+      <c r="AE14" s="9" t="n">
         <v>119.305019</v>
       </c>
-      <c r="AF14" t="inlineStr">
+      <c r="AF14" s="9" t="inlineStr">
         <is>
           <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>ATIVIDADES FINANCEIRAS, DE SEGUROS E SERVIÇOS RELACIONADOS</t>
         </is>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="7" t="n">
         <v>180</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="7" t="n">
         <v>271</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="7" t="n">
         <v>247</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="7" t="n">
         <v>344</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" s="7" t="n">
         <v>351</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="7" t="n">
         <v>393</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="J15" t="n">
+      <c r="J15" s="7" t="n">
         <v>376</v>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" s="7" t="n">
         <v>394</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="7" t="n">
         <v>1079</v>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" s="7" t="n">
         <v>1026</v>
       </c>
-      <c r="N15" t="n">
+      <c r="N15" s="7" t="n">
         <v>1352</v>
       </c>
-      <c r="O15" t="n">
+      <c r="O15" s="7" t="n">
         <v>1329</v>
       </c>
-      <c r="P15" t="n">
+      <c r="P15" s="7" t="n">
         <v>0.43906</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q15" s="7" t="n">
         <v>0.561616</v>
       </c>
-      <c r="R15" t="n">
+      <c r="R15" s="7" t="n">
         <v>0.420777</v>
       </c>
-      <c r="S15" t="n">
+      <c r="S15" s="7" t="n">
         <v>0.604287</v>
       </c>
-      <c r="T15" t="n">
+      <c r="T15" s="7" t="n">
         <v>0.5342519999999999</v>
       </c>
-      <c r="U15" t="n">
+      <c r="U15" s="7" t="n">
         <v>0.576542</v>
       </c>
-      <c r="V15" t="n">
+      <c r="V15" s="7" t="n">
         <v>0.429629</v>
       </c>
-      <c r="W15" t="n">
+      <c r="W15" s="7" t="n">
         <v>0.476789</v>
       </c>
-      <c r="X15" t="n">
+      <c r="X15" s="7" t="n">
         <v>0.489959</v>
       </c>
-      <c r="Y15" t="n">
+      <c r="Y15" s="7" t="n">
         <v>1.421805</v>
       </c>
-      <c r="Z15" t="n">
+      <c r="Z15" s="7" t="n">
         <v>1.176143</v>
       </c>
-      <c r="AA15" t="n">
+      <c r="AA15" s="7" t="n">
         <v>1.448214</v>
       </c>
-      <c r="AB15" t="n">
+      <c r="AB15" s="7" t="n">
         <v>1.496248</v>
       </c>
-      <c r="AC15" t="n">
+      <c r="AC15" s="7" t="n">
         <v>0.775025</v>
       </c>
-      <c r="AD15" t="n">
+      <c r="AD15" s="7" t="n">
         <v>1.468103</v>
       </c>
-      <c r="AE15" t="n">
+      <c r="AE15" s="7" t="n">
         <v>23.169601</v>
       </c>
-      <c r="AF15" t="inlineStr">
+      <c r="AF15" s="7" t="inlineStr">
         <is>
           <t>8/12</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>ATIVIDADES IMOBILIÁRIAS</t>
         </is>
       </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
+      <c r="C16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="9" t="n">
         <v>31</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H16" s="9" t="n">
         <v>76</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J16" s="9" t="n">
         <v>40</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="9" t="n">
         <v>180</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="9" t="n">
         <v>251</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" s="9" t="n">
         <v>236</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N16" s="9" t="n">
         <v>298</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O16" s="9" t="n">
         <v>369</v>
       </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
+      <c r="P16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="9" t="n">
         <v>0.177209</v>
       </c>
-      <c r="R16" t="n">
+      <c r="R16" s="9" t="n">
         <v>0.245831</v>
       </c>
-      <c r="S16" t="n">
+      <c r="S16" s="9" t="n">
         <v>0.76434</v>
       </c>
-      <c r="T16" t="n">
+      <c r="T16" s="9" t="n">
         <v>0.311437</v>
       </c>
-      <c r="U16" t="n">
+      <c r="U16" s="9" t="n">
         <v>0.662768</v>
       </c>
-      <c r="V16" t="n">
+      <c r="V16" s="9" t="n">
         <v>0.173736</v>
       </c>
-      <c r="W16" t="n">
+      <c r="W16" s="9" t="n">
         <v>0.314882</v>
       </c>
-      <c r="X16" t="n">
+      <c r="X16" s="9" t="n">
         <v>1.364153</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Y16" s="9" t="n">
         <v>1.903592</v>
       </c>
-      <c r="Z16" t="n">
+      <c r="Z16" s="9" t="n">
         <v>1.465834</v>
       </c>
-      <c r="AA16" t="n">
+      <c r="AA16" s="9" t="n">
         <v>1.531231</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AB16" s="9" t="n">
         <v>2.10455</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AC16" s="9" t="n">
         <v>0.8476590000000001</v>
       </c>
-      <c r="AD16" t="n">
+      <c r="AD16" s="9" t="n">
         <v>0.407622</v>
       </c>
-      <c r="AE16" t="n">
+      <c r="AE16" s="9" t="n">
         <v>47.011952</v>
       </c>
-      <c r="AF16" t="inlineStr">
+      <c r="AF16" s="9" t="inlineStr">
         <is>
           <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>ATIVIDADES PROFISSIONAIS, CIENTÍFICAS E TÉCNICAS</t>
         </is>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="7" t="n">
         <v>161</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" s="7" t="n">
         <v>156</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="7" t="n">
         <v>514</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="7" t="n">
         <v>583</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17" s="7" t="n">
         <v>671</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H17" s="7" t="n">
         <v>816</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" s="7" t="n">
         <v>533</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J17" s="7" t="n">
         <v>683</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" s="7" t="n">
         <v>625</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L17" s="7" t="n">
         <v>772</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" s="7" t="n">
         <v>1151</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N17" s="7" t="n">
         <v>1541</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O17" s="7" t="n">
         <v>1683</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P17" s="7" t="n">
         <v>0.526645</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q17" s="7" t="n">
         <v>0.414522</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R17" s="7" t="n">
         <v>1.052435</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S17" s="7" t="n">
         <v>0.88961</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T17" s="7" t="n">
         <v>0.9451889999999999</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U17" s="7" t="n">
         <v>0.9531539999999999</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V17" s="7" t="n">
         <v>0.589715</v>
       </c>
-      <c r="W17" t="n">
+      <c r="W17" s="7" t="n">
         <v>0.720955</v>
       </c>
-      <c r="X17" t="n">
+      <c r="X17" s="7" t="n">
         <v>0.632736</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y17" s="7" t="n">
         <v>0.697417</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z17" s="7" t="n">
         <v>0.8539099999999999</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA17" s="7" t="n">
         <v>0.862697</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB17" s="7" t="n">
         <v>0.873132</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AC17" s="7" t="n">
         <v>0.770163</v>
       </c>
-      <c r="AD17" t="n">
+      <c r="AD17" s="7" t="n">
         <v>1.859155</v>
       </c>
-      <c r="AE17" t="n">
+      <c r="AE17" s="7" t="n">
         <v>118.005181</v>
       </c>
-      <c r="AF17" t="inlineStr">
+      <c r="AF17" s="7" t="inlineStr">
         <is>
           <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>ATIVIDADES ADMINISTRATIVAS E SERVIÇOS COMPLEMENTARES</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="9" t="n">
         <v>1040</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" s="9" t="n">
         <v>3855</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="9" t="n">
         <v>4655</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="9" t="n">
         <v>4454</v>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" s="9" t="n">
         <v>3154</v>
       </c>
-      <c r="H18" t="n">
+      <c r="H18" s="9" t="n">
         <v>3835</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" s="9" t="n">
         <v>5791</v>
       </c>
-      <c r="J18" t="n">
+      <c r="J18" s="9" t="n">
         <v>6030</v>
       </c>
-      <c r="K18" t="n">
+      <c r="K18" s="9" t="n">
         <v>4824</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L18" s="9" t="n">
         <v>7942</v>
       </c>
-      <c r="M18" t="n">
+      <c r="M18" s="9" t="n">
         <v>9104</v>
       </c>
-      <c r="N18" t="n">
+      <c r="N18" s="9" t="n">
         <v>9786</v>
       </c>
-      <c r="O18" t="n">
+      <c r="O18" s="9" t="n">
         <v>11443</v>
       </c>
-      <c r="P18" t="n">
+      <c r="P18" s="9" t="n">
         <v>0.635027</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="Q18" s="9" t="n">
         <v>1.942517</v>
       </c>
-      <c r="R18" t="n">
+      <c r="R18" s="9" t="n">
         <v>1.797355</v>
       </c>
-      <c r="S18" t="n">
+      <c r="S18" s="9" t="n">
         <v>1.676638</v>
       </c>
-      <c r="T18" t="n">
+      <c r="T18" s="9" t="n">
         <v>1.176997</v>
       </c>
-      <c r="U18" t="n">
+      <c r="U18" s="9" t="n">
         <v>1.03618</v>
       </c>
-      <c r="V18" t="n">
+      <c r="V18" s="9" t="n">
         <v>1.609196</v>
       </c>
-      <c r="W18" t="n">
+      <c r="W18" s="9" t="n">
         <v>1.620769</v>
       </c>
-      <c r="X18" t="n">
+      <c r="X18" s="9" t="n">
         <v>1.250604</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="Y18" s="9" t="n">
         <v>1.744676</v>
       </c>
-      <c r="Z18" t="n">
+      <c r="Z18" s="9" t="n">
         <v>1.766218</v>
       </c>
-      <c r="AA18" t="n">
+      <c r="AA18" s="9" t="n">
         <v>1.498551</v>
       </c>
-      <c r="AB18" t="n">
+      <c r="AB18" s="9" t="n">
         <v>1.553833</v>
       </c>
-      <c r="AC18" t="n">
+      <c r="AC18" s="9" t="n">
         <v>1.485274</v>
       </c>
-      <c r="AD18" t="n">
+      <c r="AD18" s="9" t="n">
         <v>12.640707</v>
       </c>
-      <c r="AE18" t="n">
+      <c r="AE18" s="9" t="n">
         <v>44.082095</v>
       </c>
-      <c r="AF18" t="inlineStr">
+      <c r="AF18" s="9" t="inlineStr">
         <is>
           <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>ADMINISTRAÇÃO PÚBLICA, DEFESA E SEGURIDADE SOCIAL</t>
         </is>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="7" t="n">
         <v>3391</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" s="7" t="n">
         <v>3382</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="7" t="n">
         <v>6299</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="7" t="n">
         <v>4457</v>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" s="7" t="n">
         <v>7530</v>
       </c>
-      <c r="H19" t="n">
+      <c r="H19" s="7" t="n">
         <v>9138</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" s="7" t="n">
         <v>10318</v>
       </c>
-      <c r="J19" t="n">
+      <c r="J19" s="7" t="n">
         <v>10905</v>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" s="7" t="n">
         <v>9869</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L19" s="7" t="n">
         <v>5498</v>
       </c>
-      <c r="M19" t="n">
+      <c r="M19" s="7" t="n">
         <v>5078</v>
       </c>
-      <c r="N19" t="n">
+      <c r="N19" s="7" t="n">
         <v>6107</v>
       </c>
-      <c r="O19" t="n">
+      <c r="O19" s="7" t="n">
         <v>7211</v>
       </c>
-      <c r="P19" t="n">
+      <c r="P19" s="7" t="n">
         <v>0.336965</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="Q19" s="7" t="n">
         <v>0.248492</v>
       </c>
-      <c r="R19" t="n">
+      <c r="R19" s="7" t="n">
         <v>0.372944</v>
       </c>
-      <c r="S19" t="n">
+      <c r="S19" s="7" t="n">
         <v>0.275832</v>
       </c>
-      <c r="T19" t="n">
+      <c r="T19" s="7" t="n">
         <v>0.387277</v>
       </c>
-      <c r="U19" t="n">
+      <c r="U19" s="7" t="n">
         <v>0.414734</v>
       </c>
-      <c r="V19" t="n">
+      <c r="V19" s="7" t="n">
         <v>0.488773</v>
       </c>
-      <c r="W19" t="n">
+      <c r="W19" s="7" t="n">
         <v>0.490374</v>
       </c>
-      <c r="X19" t="n">
+      <c r="X19" s="7" t="n">
         <v>0.44233</v>
       </c>
-      <c r="Y19" t="n">
+      <c r="Y19" s="7" t="n">
         <v>0.22935</v>
       </c>
-      <c r="Z19" t="n">
+      <c r="Z19" s="7" t="n">
         <v>0.210675</v>
       </c>
-      <c r="AA19" t="n">
+      <c r="AA19" s="7" t="n">
         <v>0.237252</v>
       </c>
-      <c r="AB19" t="n">
+      <c r="AB19" s="7" t="n">
         <v>0.232131</v>
       </c>
-      <c r="AC19" t="n">
+      <c r="AC19" s="7" t="n">
         <v>0.335933</v>
       </c>
-      <c r="AD19" t="n">
+      <c r="AD19" s="7" t="n">
         <v>7.965755</v>
       </c>
-      <c r="AE19" t="n">
+      <c r="AE19" s="7" t="n">
         <v>31.156784</v>
       </c>
-      <c r="AF19" t="inlineStr">
+      <c r="AF19" s="7" t="inlineStr">
         <is>
           <t>7/12</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>EDUCAÇÃO</t>
         </is>
       </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" t="n">
+      <c r="C20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="9" t="n">
         <v>876</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="9" t="n">
         <v>1051</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="9" t="n">
         <v>1322</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" s="9" t="n">
         <v>1513</v>
       </c>
-      <c r="H20" t="n">
+      <c r="H20" s="9" t="n">
         <v>1838</v>
       </c>
-      <c r="I20" t="n">
+      <c r="I20" s="9" t="n">
         <v>1996</v>
       </c>
-      <c r="J20" t="n">
+      <c r="J20" s="9" t="n">
         <v>2265</v>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" s="9" t="n">
         <v>2588</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L20" s="9" t="n">
         <v>6932</v>
       </c>
-      <c r="M20" t="n">
+      <c r="M20" s="9" t="n">
         <v>6229</v>
       </c>
-      <c r="N20" t="n">
+      <c r="N20" s="9" t="n">
         <v>9650</v>
       </c>
-      <c r="O20" t="n">
+      <c r="O20" s="9" t="n">
         <v>12833</v>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="P20" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="Q20" t="n">
+      <c r="Q20" s="9" t="n">
         <v>1.093448</v>
       </c>
-      <c r="R20" t="n">
+      <c r="R20" s="9" t="n">
         <v>1.06935</v>
       </c>
-      <c r="S20" t="n">
+      <c r="S20" s="9" t="n">
         <v>0.906619</v>
       </c>
-      <c r="T20" t="n">
+      <c r="T20" s="9" t="n">
         <v>1.222242</v>
       </c>
-      <c r="U20" t="n">
+      <c r="U20" s="9" t="n">
         <v>1.08893</v>
       </c>
-      <c r="V20" t="n">
+      <c r="V20" s="9" t="n">
         <v>1.027401</v>
       </c>
-      <c r="W20" t="n">
+      <c r="W20" s="9" t="n">
         <v>0.91742</v>
       </c>
-      <c r="X20" t="n">
+      <c r="X20" s="9" t="n">
         <v>0.955286</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="Y20" s="9" t="n">
         <v>2.524554</v>
       </c>
-      <c r="Z20" t="n">
+      <c r="Z20" s="9" t="n">
         <v>2.630518</v>
       </c>
-      <c r="AA20" t="n">
+      <c r="AA20" s="9" t="n">
         <v>1.782708</v>
       </c>
-      <c r="AB20" t="n">
+      <c r="AB20" s="9" t="n">
         <v>2.516928</v>
       </c>
-      <c r="AC20" t="n">
+      <c r="AC20" s="9" t="n">
         <v>1.47795</v>
       </c>
-      <c r="AD20" t="n">
+      <c r="AD20" s="9" t="n">
         <v>14.176194</v>
       </c>
-      <c r="AE20" t="n">
+      <c r="AE20" s="9" t="n">
         <v>85.126947</v>
       </c>
-      <c r="AF20" t="inlineStr">
+      <c r="AF20" s="9" t="inlineStr">
         <is>
           <t>11/12</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>SAÚDE HUMANA E SERVIÇOS SOCIAIS</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="7" t="n">
         <v>576</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" s="7" t="n">
         <v>571</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="7" t="n">
         <v>637</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="7" t="n">
         <v>1834</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" s="7" t="n">
         <v>1957</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H21" s="7" t="n">
         <v>2083</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" s="7" t="n">
         <v>2073</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J21" s="7" t="n">
         <v>2515</v>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" s="7" t="n">
         <v>2777</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L21" s="7" t="n">
         <v>3172</v>
       </c>
-      <c r="M21" t="n">
+      <c r="M21" s="7" t="n">
         <v>3658</v>
       </c>
-      <c r="N21" t="n">
+      <c r="N21" s="7" t="n">
         <v>3202</v>
       </c>
-      <c r="O21" t="n">
+      <c r="O21" s="7" t="n">
         <v>3327</v>
       </c>
-      <c r="P21" t="n">
+      <c r="P21" s="7" t="n">
         <v>0.608935</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="Q21" s="7" t="n">
         <v>0.555183</v>
       </c>
-      <c r="R21" t="n">
+      <c r="R21" s="7" t="n">
         <v>0.538399</v>
       </c>
-      <c r="S21" t="n">
+      <c r="S21" s="7" t="n">
         <v>1.469437</v>
       </c>
-      <c r="T21" t="n">
+      <c r="T21" s="7" t="n">
         <v>1.489968</v>
       </c>
-      <c r="U21" t="n">
+      <c r="U21" s="7" t="n">
         <v>1.353741</v>
       </c>
-      <c r="V21" t="n">
+      <c r="V21" s="7" t="n">
         <v>1.194519</v>
       </c>
-      <c r="W21" t="n">
+      <c r="W21" s="7" t="n">
         <v>1.133038</v>
       </c>
-      <c r="X21" t="n">
+      <c r="X21" s="7" t="n">
         <v>1.09314</v>
       </c>
-      <c r="Y21" t="n">
+      <c r="Y21" s="7" t="n">
         <v>1.371292</v>
       </c>
-      <c r="Z21" t="n">
+      <c r="Z21" s="7" t="n">
         <v>1.33919</v>
       </c>
-      <c r="AA21" t="n">
+      <c r="AA21" s="7" t="n">
         <v>0.900875</v>
       </c>
-      <c r="AB21" t="n">
+      <c r="AB21" s="7" t="n">
         <v>0.853013</v>
       </c>
-      <c r="AC21" t="n">
+      <c r="AC21" s="7" t="n">
         <v>1.069287</v>
       </c>
-      <c r="AD21" t="n">
+      <c r="AD21" s="7" t="n">
         <v>3.675228</v>
       </c>
-      <c r="AE21" t="n">
+      <c r="AE21" s="7" t="n">
         <v>4.886507</v>
       </c>
-      <c r="AF21" t="inlineStr">
+      <c r="AF21" s="7" t="inlineStr">
         <is>
           <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>ARTES, CULTURA, ESPORTE E RECREAÇÃO</t>
         </is>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="9" t="n">
         <v>86</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" s="9" t="n">
         <v>115</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="9" t="n">
         <v>93</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="9" t="n">
         <v>131</v>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" s="9" t="n">
         <v>141</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H22" s="9" t="n">
         <v>207</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I22" s="9" t="n">
         <v>213</v>
       </c>
-      <c r="J22" t="n">
+      <c r="J22" s="9" t="n">
         <v>256</v>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" s="9" t="n">
         <v>260</v>
       </c>
-      <c r="L22" t="n">
+      <c r="L22" s="9" t="n">
         <v>290</v>
       </c>
-      <c r="M22" t="n">
+      <c r="M22" s="9" t="n">
         <v>350</v>
       </c>
-      <c r="N22" t="n">
+      <c r="N22" s="9" t="n">
         <v>445</v>
       </c>
-      <c r="O22" t="n">
+      <c r="O22" s="9" t="n">
         <v>575</v>
       </c>
-      <c r="P22" t="n">
+      <c r="P22" s="9" t="n">
         <v>0.567574</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="Q22" s="9" t="n">
         <v>0.696394</v>
       </c>
-      <c r="R22" t="n">
+      <c r="R22" s="9" t="n">
         <v>0.510064</v>
       </c>
-      <c r="S22" t="n">
+      <c r="S22" s="9" t="n">
         <v>0.6834519999999999</v>
       </c>
-      <c r="T22" t="n">
+      <c r="T22" s="9" t="n">
         <v>0.721378</v>
       </c>
-      <c r="U22" t="n">
+      <c r="U22" s="9" t="n">
         <v>0.881933</v>
       </c>
-      <c r="V22" t="n">
+      <c r="V22" s="9" t="n">
         <v>0.983508</v>
       </c>
-      <c r="W22" t="n">
+      <c r="W22" s="9" t="n">
         <v>0.8218800000000001</v>
       </c>
-      <c r="X22" t="n">
+      <c r="X22" s="9" t="n">
         <v>0.857727</v>
       </c>
-      <c r="Y22" t="n">
+      <c r="Y22" s="9" t="n">
         <v>1.277689</v>
       </c>
-      <c r="Z22" t="n">
+      <c r="Z22" s="9" t="n">
         <v>1.61837</v>
       </c>
-      <c r="AA22" t="n">
+      <c r="AA22" s="9" t="n">
         <v>1.362921</v>
       </c>
-      <c r="AB22" t="n">
+      <c r="AB22" s="9" t="n">
         <v>1.419695</v>
       </c>
-      <c r="AC22" t="n">
+      <c r="AC22" s="9" t="n">
         <v>0.954045</v>
       </c>
-      <c r="AD22" t="n">
+      <c r="AD22" s="9" t="n">
         <v>0.635184</v>
       </c>
-      <c r="AE22" t="n">
+      <c r="AE22" s="9" t="n">
         <v>98.275862</v>
       </c>
-      <c r="AF22" t="inlineStr">
+      <c r="AF22" s="9" t="inlineStr">
         <is>
           <t>11/12</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>OUTRAS ATIVIDADES DE SERVIÇOS</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="7" t="n">
         <v>609</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" s="7" t="n">
         <v>675</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="7" t="n">
         <v>756</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="7" t="n">
         <v>518</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" s="7" t="n">
         <v>544</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H23" s="7" t="n">
         <v>579</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" s="7" t="n">
         <v>627</v>
       </c>
-      <c r="J23" t="n">
+      <c r="J23" s="7" t="n">
         <v>616</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K23" s="7" t="n">
         <v>844</v>
       </c>
-      <c r="L23" t="n">
+      <c r="L23" s="7" t="n">
         <v>895</v>
       </c>
-      <c r="M23" t="n">
+      <c r="M23" s="7" t="n">
         <v>1049</v>
       </c>
-      <c r="N23" t="n">
+      <c r="N23" s="7" t="n">
         <v>849</v>
       </c>
-      <c r="O23" t="n">
+      <c r="O23" s="7" t="n">
         <v>1050</v>
       </c>
-      <c r="P23" t="n">
+      <c r="P23" s="7" t="n">
         <v>0.69369</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q23" s="7" t="n">
         <v>0.633938</v>
       </c>
-      <c r="R23" t="n">
+      <c r="R23" s="7" t="n">
         <v>0.703484</v>
       </c>
-      <c r="S23" t="n">
+      <c r="S23" s="7" t="n">
         <v>0.498673</v>
       </c>
-      <c r="T23" t="n">
+      <c r="T23" s="7" t="n">
         <v>0.5738529999999999</v>
       </c>
-      <c r="U23" t="n">
+      <c r="U23" s="7" t="n">
         <v>0.557488</v>
       </c>
-      <c r="V23" t="n">
+      <c r="V23" s="7" t="n">
         <v>0.628477</v>
       </c>
-      <c r="W23" t="n">
+      <c r="W23" s="7" t="n">
         <v>0.529511</v>
       </c>
-      <c r="X23" t="n">
+      <c r="X23" s="7" t="n">
         <v>0.764243</v>
       </c>
-      <c r="Y23" t="n">
+      <c r="Y23" s="7" t="n">
         <v>0.836153</v>
       </c>
-      <c r="Z23" t="n">
+      <c r="Z23" s="7" t="n">
         <v>0.964286</v>
       </c>
-      <c r="AA23" t="n">
+      <c r="AA23" s="7" t="n">
         <v>0.5978250000000001</v>
       </c>
-      <c r="AB23" t="n">
+      <c r="AB23" s="7" t="n">
         <v>0.735486</v>
       </c>
-      <c r="AC23" t="n">
+      <c r="AC23" s="7" t="n">
         <v>0.670547</v>
       </c>
-      <c r="AD23" t="n">
+      <c r="AD23" s="7" t="n">
         <v>1.159901</v>
       </c>
-      <c r="AE23" t="n">
+      <c r="AE23" s="7" t="n">
         <v>17.318436</v>
       </c>
-      <c r="AF23" t="inlineStr">
+      <c r="AF23" s="7" t="inlineStr">
         <is>
           <t>9/12</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>SERVIÇOS DOMÉSTICOS</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="H24" t="n">
+      <c r="H24" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
+      <c r="I24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="K24" t="n">
+      <c r="K24" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L24" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="n">
+      <c r="M24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="9" t="n">
         <v>0.655625</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="Q24" s="9" t="n">
         <v>0.386525</v>
       </c>
-      <c r="R24" t="n">
+      <c r="R24" s="9" t="n">
         <v>0.275496</v>
       </c>
-      <c r="S24" t="n">
+      <c r="S24" s="9" t="n">
         <v>0.48443</v>
       </c>
-      <c r="T24" t="n">
+      <c r="T24" s="9" t="n">
         <v>0.702868</v>
       </c>
-      <c r="U24" t="n">
+      <c r="U24" s="9" t="n">
         <v>0.666344</v>
       </c>
-      <c r="V24" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" t="n">
+      <c r="V24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" s="9" t="n">
         <v>1.434728</v>
       </c>
-      <c r="X24" t="n">
+      <c r="X24" s="9" t="n">
         <v>2.656186</v>
       </c>
-      <c r="Y24" t="n">
+      <c r="Y24" s="9" t="n">
         <v>2.50273</v>
       </c>
-      <c r="Z24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC24" t="n">
+      <c r="Z24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="9" t="n">
         <v>0.751149</v>
       </c>
-      <c r="AD24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE24" t="n">
+      <c r="AD24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="9" t="n">
         <v>-100</v>
       </c>
-      <c r="AF24" t="inlineStr">
+      <c r="AF24" s="9" t="inlineStr">
         <is>
           <t>4/12</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>ORGANISMOS INTERNACIONAIS E OUTRAS INSTITUIÇÕES EXTRATERRITORIAIS</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="n">
+      <c r="D25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="7" t="n">
         <v>12.331998</v>
       </c>
-      <c r="Q25" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" t="n">
-        <v>0</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0</v>
-      </c>
-      <c r="V25" t="n">
-        <v>0</v>
-      </c>
-      <c r="W25" t="n">
-        <v>0</v>
-      </c>
-      <c r="X25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC25" t="n">
+      <c r="Q25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="7" t="n">
         <v>0.948615</v>
       </c>
-      <c r="AD25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE25" t="inlineStr">
+      <c r="AD25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="AF25" t="inlineStr">
+      <c r="AF25" s="7" t="inlineStr">
         <is>
           <t>0/12</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:AF1"/>
+    <mergeCell ref="A2:AF2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>